<commit_message>
refined intraday and swing strategies
</commit_message>
<xml_diff>
--- a/Nifty_Trading_Journal.xlsx
+++ b/Nifty_Trading_Journal.xlsx
@@ -19,11 +19,14 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <numFmts count="2">
+  <numFmts count="5">
     <numFmt numFmtId="164" formatCode="0.0%"/>
     <numFmt numFmtId="165" formatCode="₹#,##0;(₹#,##0);&quot;-&quot;"/>
+    <numFmt numFmtId="166" formatCode="₹#,##0"/>
+    <numFmt numFmtId="167" formatCode="DD-MMM-YY"/>
+    <numFmt numFmtId="168" formatCode="yyyy-mm-dd"/>
   </numFmts>
-  <fonts count="14">
+  <fonts count="18">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -103,8 +106,29 @@
       <color rgb="00999999"/>
       <sz val="10"/>
     </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
+      <sz val="10"/>
+    </font>
   </fonts>
-  <fills count="18">
+  <fills count="25">
     <fill>
       <patternFill/>
     </fill>
@@ -207,8 +231,43 @@
         <bgColor rgb="006C3483"/>
       </patternFill>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00C55A11"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00833C00"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00375623"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00E2EFDA"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E79"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00DDEEFF"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00FFFFFF"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="2">
+  <borders count="11">
     <border>
       <left/>
       <right/>
@@ -230,11 +289,113 @@
         <color rgb="00CCCCCC"/>
       </bottom>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00CCCCCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="00CCCCCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00CCCCCC"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color rgb="00808080"/>
+      </left>
+      <right style="thin">
+        <color rgb="00808080"/>
+      </right>
+      <top style="thin">
+        <color rgb="00808080"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00808080"/>
+      </bottom>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00808080"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00808080"/>
+      </right>
+      <top style="thin">
+        <color rgb="00808080"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin">
+        <color rgb="00808080"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00808080"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color rgb="00808080"/>
+      </right>
+      <top style="thin">
+        <color rgb="00808080"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="00808080"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="66">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -342,6 +503,82 @@
     </xf>
     <xf numFmtId="0" fontId="13" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="18" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="19" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="10" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="14" fillId="20" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="21" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="21" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="16" fillId="21" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="22" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="23" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="164" fontId="16" fillId="23" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="166" fontId="16" fillId="23" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="19" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="0" borderId="6" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="167" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="21" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="167" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="23" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="24" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="6" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -734,11 +971,11 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:R54"/>
+  <dimension ref="A1:S54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
-    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="11" customWidth="1" min="2" max="2"/>
     <col width="8" customWidth="1" min="3" max="3"/>
     <col width="10" customWidth="1" min="4" max="4"/>
     <col width="10" customWidth="1" min="5" max="5"/>
@@ -778,157 +1015,270 @@
           <t>Date</t>
         </is>
       </c>
-      <c r="B4" s="3" t="inlineStr">
+      <c r="B4" s="38" t="inlineStr">
+        <is>
+          <t>Strategy</t>
+        </is>
+      </c>
+      <c r="C4" s="3" t="inlineStr">
         <is>
           <t>Day</t>
         </is>
       </c>
-      <c r="C4" s="3" t="inlineStr">
+      <c r="D4" s="3" t="inlineStr">
         <is>
           <t>Time
 Entry</t>
         </is>
       </c>
-      <c r="D4" s="3" t="inlineStr">
+      <c r="E4" s="3" t="inlineStr">
         <is>
           <t>Expiry</t>
         </is>
       </c>
-      <c r="E4" s="3" t="inlineStr">
+      <c r="F4" s="3" t="inlineStr">
         <is>
           <t>Trade
 Type</t>
         </is>
       </c>
-      <c r="F4" s="3" t="inlineStr">
+      <c r="G4" s="3" t="inlineStr">
         <is>
           <t>Strike</t>
         </is>
       </c>
-      <c r="G4" s="3" t="inlineStr">
+      <c r="H4" s="3" t="inlineStr">
         <is>
           <t>Entry
 Price ₹</t>
         </is>
       </c>
-      <c r="H4" s="3" t="inlineStr">
+      <c r="I4" s="3" t="inlineStr">
         <is>
           <t>Exit
 Price ₹</t>
         </is>
       </c>
-      <c r="I4" s="3" t="inlineStr">
+      <c r="J4" s="3" t="inlineStr">
         <is>
           <t>Stop
 Loss ₹</t>
         </is>
       </c>
-      <c r="J4" s="3" t="inlineStr">
+      <c r="K4" s="3" t="inlineStr">
         <is>
           <t>Target
 1 ₹</t>
         </is>
       </c>
-      <c r="K4" s="3" t="inlineStr">
+      <c r="L4" s="3" t="inlineStr">
         <is>
           <t>Target
 2 ₹</t>
         </is>
       </c>
-      <c r="L4" s="3" t="inlineStr">
+      <c r="M4" s="3" t="inlineStr">
         <is>
           <t>Lots</t>
         </is>
       </c>
-      <c r="M4" s="3" t="inlineStr">
+      <c r="N4" s="3" t="inlineStr">
         <is>
           <t>P&amp;L ₹</t>
         </is>
       </c>
-      <c r="N4" s="3" t="inlineStr">
+      <c r="O4" s="3" t="inlineStr">
         <is>
           <t>Result</t>
         </is>
       </c>
-      <c r="O4" s="3" t="inlineStr">
+      <c r="P4" s="3" t="inlineStr">
         <is>
           <t>R:R
 Achieved</t>
         </is>
       </c>
-      <c r="P4" s="3" t="inlineStr">
+      <c r="Q4" s="3" t="inlineStr">
         <is>
           <t>Filters
 Followed</t>
         </is>
       </c>
-      <c r="Q4" s="3" t="inlineStr">
+      <c r="R4" s="3" t="inlineStr">
         <is>
           <t>Market
 Bias</t>
         </is>
       </c>
-      <c r="R4" s="3" t="inlineStr">
+      <c r="S4" s="3" t="inlineStr">
         <is>
           <t>Notes / Lessons</t>
         </is>
       </c>
     </row>
     <row r="5">
-      <c r="A5" s="4" t="n"/>
-      <c r="B5" s="4" t="n"/>
-      <c r="C5" s="4" t="n"/>
-      <c r="D5" s="4" t="n"/>
-      <c r="E5" s="4" t="n"/>
-      <c r="F5" s="4" t="n"/>
-      <c r="G5" s="4" t="n"/>
-      <c r="H5" s="4" t="n"/>
-      <c r="I5" s="4" t="n"/>
-      <c r="J5" s="4" t="n"/>
-      <c r="K5" s="4" t="n"/>
-      <c r="L5" s="4" t="n"/>
-      <c r="M5" s="4">
-        <f>(H5-G5)*L5*25</f>
-        <v/>
-      </c>
-      <c r="N5" s="4" t="n"/>
-      <c r="O5" s="4">
-        <f>IFERROR((H5-G5)/(G5-I5),"—")</f>
-        <v/>
-      </c>
-      <c r="P5" s="4" t="n"/>
-      <c r="Q5" s="4" t="n"/>
-      <c r="R5" s="5" t="n"/>
+      <c r="A5" s="60" t="n">
+        <v>46154</v>
+      </c>
+      <c r="B5" s="56" t="inlineStr">
+        <is>
+          <t>Intraday</t>
+        </is>
+      </c>
+      <c r="C5" s="57" t="inlineStr">
+        <is>
+          <t>Tuesday</t>
+        </is>
+      </c>
+      <c r="D5" s="57" t="inlineStr">
+        <is>
+          <t>10:10</t>
+        </is>
+      </c>
+      <c r="E5" s="57" t="inlineStr">
+        <is>
+          <t>Weekly</t>
+        </is>
+      </c>
+      <c r="F5" s="57" t="inlineStr">
+        <is>
+          <t>Put Sell</t>
+        </is>
+      </c>
+      <c r="G5" s="57" t="inlineStr">
+        <is>
+          <t>23800 PE</t>
+        </is>
+      </c>
+      <c r="H5" s="57" t="n">
+        <v>160.15</v>
+      </c>
+      <c r="I5" s="57" t="n">
+        <v>171.25</v>
+      </c>
+      <c r="J5" s="57" t="n">
+        <v>190</v>
+      </c>
+      <c r="K5" s="57" t="n">
+        <v>161.25</v>
+      </c>
+      <c r="L5" s="57" t="n"/>
+      <c r="M5" s="57" t="n">
+        <v>1</v>
+      </c>
+      <c r="N5" s="57">
+        <f>(I5-H5)*M5*65</f>
+        <v/>
+      </c>
+      <c r="O5" s="58" t="inlineStr">
+        <is>
+          <t>Profit</t>
+        </is>
+      </c>
+      <c r="P5" s="57">
+        <f>IFERROR((I5-H5)/(H5-J5),"—")</f>
+        <v/>
+      </c>
+      <c r="Q5" s="57" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R5" s="57" t="inlineStr">
+        <is>
+          <t>Bullish</t>
+        </is>
+      </c>
+      <c r="S5" s="59" t="inlineStr">
+        <is>
+          <t>Reversal trade at 23800 retest. Booked early at ~10 pts. RSI oversold bounce + theta decay on expiry day.</t>
+        </is>
+      </c>
     </row>
     <row r="6">
-      <c r="A6" s="6" t="n"/>
-      <c r="B6" s="6" t="n"/>
-      <c r="C6" s="6" t="n"/>
-      <c r="D6" s="6" t="n"/>
-      <c r="E6" s="6" t="n"/>
-      <c r="F6" s="6" t="n"/>
-      <c r="G6" s="6" t="n"/>
-      <c r="H6" s="6" t="n"/>
-      <c r="I6" s="6" t="n"/>
-      <c r="J6" s="6" t="n"/>
-      <c r="K6" s="6" t="n"/>
-      <c r="L6" s="6" t="n"/>
-      <c r="M6" s="6">
-        <f>(H6-G6)*L6*25</f>
-        <v/>
-      </c>
-      <c r="N6" s="6" t="n"/>
-      <c r="O6" s="6">
-        <f>IFERROR((H6-G6)/(G6-I6),"—")</f>
-        <v/>
-      </c>
-      <c r="P6" s="6" t="n"/>
-      <c r="Q6" s="6" t="n"/>
-      <c r="R6" s="7" t="n"/>
+      <c r="A6" s="61" t="n">
+        <v>46155</v>
+      </c>
+      <c r="B6" s="62" t="inlineStr">
+        <is>
+          <t>Swing</t>
+        </is>
+      </c>
+      <c r="C6" s="63" t="inlineStr">
+        <is>
+          <t>Wednesday</t>
+        </is>
+      </c>
+      <c r="D6" s="63" t="inlineStr">
+        <is>
+          <t>12:02</t>
+        </is>
+      </c>
+      <c r="E6" s="63" t="inlineStr">
+        <is>
+          <t>Monthly</t>
+        </is>
+      </c>
+      <c r="F6" s="63" t="inlineStr">
+        <is>
+          <t>PE Buy</t>
+        </is>
+      </c>
+      <c r="G6" s="63" t="inlineStr">
+        <is>
+          <t>24000 PE</t>
+        </is>
+      </c>
+      <c r="H6" s="63" t="n">
+        <v>618.9</v>
+      </c>
+      <c r="I6" s="63" t="n">
+        <v>0</v>
+      </c>
+      <c r="J6" s="63" t="n">
+        <v>570</v>
+      </c>
+      <c r="K6" s="63" t="n">
+        <v>783</v>
+      </c>
+      <c r="L6" s="63" t="n">
+        <v>1044</v>
+      </c>
+      <c r="M6" s="63" t="n">
+        <v>1</v>
+      </c>
+      <c r="N6" s="63">
+        <f>(I6-H6)*M6*25</f>
+        <v/>
+      </c>
+      <c r="O6" s="64" t="inlineStr">
+        <is>
+          <t>Open</t>
+        </is>
+      </c>
+      <c r="P6" s="63">
+        <f>IFERROR((I6-H6)/(H6-J6),"—")</f>
+        <v/>
+      </c>
+      <c r="Q6" s="63" t="inlineStr">
+        <is>
+          <t>Yes</t>
+        </is>
+      </c>
+      <c r="R6" s="63" t="inlineStr">
+        <is>
+          <t>Bearish</t>
+        </is>
+      </c>
+      <c r="S6" s="65" t="inlineStr">
+        <is>
+          <t>Deep ITM monthly PE swing. All 3 HTF bearish. Entry near 23500 ATM. Holding overnight. Grade B setup.</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="4" t="n"/>
-      <c r="B7" s="4" t="n"/>
+      <c r="B7" s="39" t="n"/>
       <c r="C7" s="4" t="n"/>
       <c r="D7" s="4" t="n"/>
       <c r="E7" s="4" t="n"/>
@@ -939,22 +1289,23 @@
       <c r="J7" s="4" t="n"/>
       <c r="K7" s="4" t="n"/>
       <c r="L7" s="4" t="n"/>
-      <c r="M7" s="4">
-        <f>(H7-G7)*L7*25</f>
-        <v/>
-      </c>
-      <c r="N7" s="4" t="n"/>
-      <c r="O7" s="4">
+      <c r="M7" s="4" t="n"/>
+      <c r="N7" s="4">
+        <f>(H7-G7)*L7*65</f>
+        <v/>
+      </c>
+      <c r="O7" s="4" t="n"/>
+      <c r="P7" s="4">
         <f>IFERROR((H7-G7)/(G7-I7),"—")</f>
         <v/>
       </c>
-      <c r="P7" s="4" t="n"/>
       <c r="Q7" s="4" t="n"/>
-      <c r="R7" s="5" t="n"/>
+      <c r="R7" s="4" t="n"/>
+      <c r="S7" s="5" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="n"/>
-      <c r="B8" s="6" t="n"/>
+      <c r="B8" s="39" t="n"/>
       <c r="C8" s="6" t="n"/>
       <c r="D8" s="6" t="n"/>
       <c r="E8" s="6" t="n"/>
@@ -965,22 +1316,23 @@
       <c r="J8" s="6" t="n"/>
       <c r="K8" s="6" t="n"/>
       <c r="L8" s="6" t="n"/>
-      <c r="M8" s="6">
-        <f>(H8-G8)*L8*25</f>
-        <v/>
-      </c>
-      <c r="N8" s="6" t="n"/>
-      <c r="O8" s="6">
+      <c r="M8" s="6" t="n"/>
+      <c r="N8" s="6">
+        <f>(H8-G8)*L8*65</f>
+        <v/>
+      </c>
+      <c r="O8" s="6" t="n"/>
+      <c r="P8" s="6">
         <f>IFERROR((H8-G8)/(G8-I8),"—")</f>
         <v/>
       </c>
-      <c r="P8" s="6" t="n"/>
       <c r="Q8" s="6" t="n"/>
-      <c r="R8" s="7" t="n"/>
+      <c r="R8" s="6" t="n"/>
+      <c r="S8" s="7" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="4" t="n"/>
-      <c r="B9" s="4" t="n"/>
+      <c r="B9" s="39" t="n"/>
       <c r="C9" s="4" t="n"/>
       <c r="D9" s="4" t="n"/>
       <c r="E9" s="4" t="n"/>
@@ -991,22 +1343,23 @@
       <c r="J9" s="4" t="n"/>
       <c r="K9" s="4" t="n"/>
       <c r="L9" s="4" t="n"/>
-      <c r="M9" s="4">
-        <f>(H9-G9)*L9*25</f>
-        <v/>
-      </c>
-      <c r="N9" s="4" t="n"/>
-      <c r="O9" s="4">
+      <c r="M9" s="4" t="n"/>
+      <c r="N9" s="4">
+        <f>(H9-G9)*L9*65</f>
+        <v/>
+      </c>
+      <c r="O9" s="4" t="n"/>
+      <c r="P9" s="4">
         <f>IFERROR((H9-G9)/(G9-I9),"—")</f>
         <v/>
       </c>
-      <c r="P9" s="4" t="n"/>
       <c r="Q9" s="4" t="n"/>
-      <c r="R9" s="5" t="n"/>
+      <c r="R9" s="4" t="n"/>
+      <c r="S9" s="5" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="n"/>
-      <c r="B10" s="6" t="n"/>
+      <c r="B10" s="39" t="n"/>
       <c r="C10" s="6" t="n"/>
       <c r="D10" s="6" t="n"/>
       <c r="E10" s="6" t="n"/>
@@ -1017,22 +1370,23 @@
       <c r="J10" s="6" t="n"/>
       <c r="K10" s="6" t="n"/>
       <c r="L10" s="6" t="n"/>
-      <c r="M10" s="6">
-        <f>(H10-G10)*L10*25</f>
-        <v/>
-      </c>
-      <c r="N10" s="6" t="n"/>
-      <c r="O10" s="6">
+      <c r="M10" s="6" t="n"/>
+      <c r="N10" s="6">
+        <f>(H10-G10)*L10*65</f>
+        <v/>
+      </c>
+      <c r="O10" s="6" t="n"/>
+      <c r="P10" s="6">
         <f>IFERROR((H10-G10)/(G10-I10),"—")</f>
         <v/>
       </c>
-      <c r="P10" s="6" t="n"/>
       <c r="Q10" s="6" t="n"/>
-      <c r="R10" s="7" t="n"/>
+      <c r="R10" s="6" t="n"/>
+      <c r="S10" s="7" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="4" t="n"/>
-      <c r="B11" s="4" t="n"/>
+      <c r="B11" s="39" t="n"/>
       <c r="C11" s="4" t="n"/>
       <c r="D11" s="4" t="n"/>
       <c r="E11" s="4" t="n"/>
@@ -1043,22 +1397,23 @@
       <c r="J11" s="4" t="n"/>
       <c r="K11" s="4" t="n"/>
       <c r="L11" s="4" t="n"/>
-      <c r="M11" s="4">
-        <f>(H11-G11)*L11*25</f>
-        <v/>
-      </c>
-      <c r="N11" s="4" t="n"/>
-      <c r="O11" s="4">
+      <c r="M11" s="4" t="n"/>
+      <c r="N11" s="4">
+        <f>(H11-G11)*L11*65</f>
+        <v/>
+      </c>
+      <c r="O11" s="4" t="n"/>
+      <c r="P11" s="4">
         <f>IFERROR((H11-G11)/(G11-I11),"—")</f>
         <v/>
       </c>
-      <c r="P11" s="4" t="n"/>
       <c r="Q11" s="4" t="n"/>
-      <c r="R11" s="5" t="n"/>
+      <c r="R11" s="4" t="n"/>
+      <c r="S11" s="5" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="n"/>
-      <c r="B12" s="6" t="n"/>
+      <c r="B12" s="39" t="n"/>
       <c r="C12" s="6" t="n"/>
       <c r="D12" s="6" t="n"/>
       <c r="E12" s="6" t="n"/>
@@ -1069,22 +1424,23 @@
       <c r="J12" s="6" t="n"/>
       <c r="K12" s="6" t="n"/>
       <c r="L12" s="6" t="n"/>
-      <c r="M12" s="6">
-        <f>(H12-G12)*L12*25</f>
-        <v/>
-      </c>
-      <c r="N12" s="6" t="n"/>
-      <c r="O12" s="6">
+      <c r="M12" s="6" t="n"/>
+      <c r="N12" s="6">
+        <f>(H12-G12)*L12*65</f>
+        <v/>
+      </c>
+      <c r="O12" s="6" t="n"/>
+      <c r="P12" s="6">
         <f>IFERROR((H12-G12)/(G12-I12),"—")</f>
         <v/>
       </c>
-      <c r="P12" s="6" t="n"/>
       <c r="Q12" s="6" t="n"/>
-      <c r="R12" s="7" t="n"/>
+      <c r="R12" s="6" t="n"/>
+      <c r="S12" s="7" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="4" t="n"/>
-      <c r="B13" s="4" t="n"/>
+      <c r="B13" s="39" t="n"/>
       <c r="C13" s="4" t="n"/>
       <c r="D13" s="4" t="n"/>
       <c r="E13" s="4" t="n"/>
@@ -1095,22 +1451,23 @@
       <c r="J13" s="4" t="n"/>
       <c r="K13" s="4" t="n"/>
       <c r="L13" s="4" t="n"/>
-      <c r="M13" s="4">
-        <f>(H13-G13)*L13*25</f>
-        <v/>
-      </c>
-      <c r="N13" s="4" t="n"/>
-      <c r="O13" s="4">
+      <c r="M13" s="4" t="n"/>
+      <c r="N13" s="4">
+        <f>(H13-G13)*L13*65</f>
+        <v/>
+      </c>
+      <c r="O13" s="4" t="n"/>
+      <c r="P13" s="4">
         <f>IFERROR((H13-G13)/(G13-I13),"—")</f>
         <v/>
       </c>
-      <c r="P13" s="4" t="n"/>
       <c r="Q13" s="4" t="n"/>
-      <c r="R13" s="5" t="n"/>
+      <c r="R13" s="4" t="n"/>
+      <c r="S13" s="5" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="6" t="n"/>
-      <c r="B14" s="6" t="n"/>
+      <c r="B14" s="39" t="n"/>
       <c r="C14" s="6" t="n"/>
       <c r="D14" s="6" t="n"/>
       <c r="E14" s="6" t="n"/>
@@ -1121,22 +1478,23 @@
       <c r="J14" s="6" t="n"/>
       <c r="K14" s="6" t="n"/>
       <c r="L14" s="6" t="n"/>
-      <c r="M14" s="6">
-        <f>(H14-G14)*L14*25</f>
-        <v/>
-      </c>
-      <c r="N14" s="6" t="n"/>
-      <c r="O14" s="6">
+      <c r="M14" s="6" t="n"/>
+      <c r="N14" s="6">
+        <f>(H14-G14)*L14*65</f>
+        <v/>
+      </c>
+      <c r="O14" s="6" t="n"/>
+      <c r="P14" s="6">
         <f>IFERROR((H14-G14)/(G14-I14),"—")</f>
         <v/>
       </c>
-      <c r="P14" s="6" t="n"/>
       <c r="Q14" s="6" t="n"/>
-      <c r="R14" s="7" t="n"/>
+      <c r="R14" s="6" t="n"/>
+      <c r="S14" s="7" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="4" t="n"/>
-      <c r="B15" s="4" t="n"/>
+      <c r="B15" s="39" t="n"/>
       <c r="C15" s="4" t="n"/>
       <c r="D15" s="4" t="n"/>
       <c r="E15" s="4" t="n"/>
@@ -1147,22 +1505,23 @@
       <c r="J15" s="4" t="n"/>
       <c r="K15" s="4" t="n"/>
       <c r="L15" s="4" t="n"/>
-      <c r="M15" s="4">
-        <f>(H15-G15)*L15*25</f>
-        <v/>
-      </c>
-      <c r="N15" s="4" t="n"/>
-      <c r="O15" s="4">
+      <c r="M15" s="4" t="n"/>
+      <c r="N15" s="4">
+        <f>(H15-G15)*L15*65</f>
+        <v/>
+      </c>
+      <c r="O15" s="4" t="n"/>
+      <c r="P15" s="4">
         <f>IFERROR((H15-G15)/(G15-I15),"—")</f>
         <v/>
       </c>
-      <c r="P15" s="4" t="n"/>
       <c r="Q15" s="4" t="n"/>
-      <c r="R15" s="5" t="n"/>
+      <c r="R15" s="4" t="n"/>
+      <c r="S15" s="5" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="n"/>
-      <c r="B16" s="6" t="n"/>
+      <c r="B16" s="39" t="n"/>
       <c r="C16" s="6" t="n"/>
       <c r="D16" s="6" t="n"/>
       <c r="E16" s="6" t="n"/>
@@ -1173,22 +1532,23 @@
       <c r="J16" s="6" t="n"/>
       <c r="K16" s="6" t="n"/>
       <c r="L16" s="6" t="n"/>
-      <c r="M16" s="6">
-        <f>(H16-G16)*L16*25</f>
-        <v/>
-      </c>
-      <c r="N16" s="6" t="n"/>
-      <c r="O16" s="6">
+      <c r="M16" s="6" t="n"/>
+      <c r="N16" s="6">
+        <f>(H16-G16)*L16*65</f>
+        <v/>
+      </c>
+      <c r="O16" s="6" t="n"/>
+      <c r="P16" s="6">
         <f>IFERROR((H16-G16)/(G16-I16),"—")</f>
         <v/>
       </c>
-      <c r="P16" s="6" t="n"/>
       <c r="Q16" s="6" t="n"/>
-      <c r="R16" s="7" t="n"/>
+      <c r="R16" s="6" t="n"/>
+      <c r="S16" s="7" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="4" t="n"/>
-      <c r="B17" s="4" t="n"/>
+      <c r="B17" s="39" t="n"/>
       <c r="C17" s="4" t="n"/>
       <c r="D17" s="4" t="n"/>
       <c r="E17" s="4" t="n"/>
@@ -1199,22 +1559,23 @@
       <c r="J17" s="4" t="n"/>
       <c r="K17" s="4" t="n"/>
       <c r="L17" s="4" t="n"/>
-      <c r="M17" s="4">
-        <f>(H17-G17)*L17*25</f>
-        <v/>
-      </c>
-      <c r="N17" s="4" t="n"/>
-      <c r="O17" s="4">
+      <c r="M17" s="4" t="n"/>
+      <c r="N17" s="4">
+        <f>(H17-G17)*L17*65</f>
+        <v/>
+      </c>
+      <c r="O17" s="4" t="n"/>
+      <c r="P17" s="4">
         <f>IFERROR((H17-G17)/(G17-I17),"—")</f>
         <v/>
       </c>
-      <c r="P17" s="4" t="n"/>
       <c r="Q17" s="4" t="n"/>
-      <c r="R17" s="5" t="n"/>
+      <c r="R17" s="4" t="n"/>
+      <c r="S17" s="5" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="n"/>
-      <c r="B18" s="6" t="n"/>
+      <c r="B18" s="39" t="n"/>
       <c r="C18" s="6" t="n"/>
       <c r="D18" s="6" t="n"/>
       <c r="E18" s="6" t="n"/>
@@ -1225,22 +1586,23 @@
       <c r="J18" s="6" t="n"/>
       <c r="K18" s="6" t="n"/>
       <c r="L18" s="6" t="n"/>
-      <c r="M18" s="6">
-        <f>(H18-G18)*L18*25</f>
-        <v/>
-      </c>
-      <c r="N18" s="6" t="n"/>
-      <c r="O18" s="6">
+      <c r="M18" s="6" t="n"/>
+      <c r="N18" s="6">
+        <f>(H18-G18)*L18*65</f>
+        <v/>
+      </c>
+      <c r="O18" s="6" t="n"/>
+      <c r="P18" s="6">
         <f>IFERROR((H18-G18)/(G18-I18),"—")</f>
         <v/>
       </c>
-      <c r="P18" s="6" t="n"/>
       <c r="Q18" s="6" t="n"/>
-      <c r="R18" s="7" t="n"/>
+      <c r="R18" s="6" t="n"/>
+      <c r="S18" s="7" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="4" t="n"/>
-      <c r="B19" s="4" t="n"/>
+      <c r="B19" s="39" t="n"/>
       <c r="C19" s="4" t="n"/>
       <c r="D19" s="4" t="n"/>
       <c r="E19" s="4" t="n"/>
@@ -1251,22 +1613,23 @@
       <c r="J19" s="4" t="n"/>
       <c r="K19" s="4" t="n"/>
       <c r="L19" s="4" t="n"/>
-      <c r="M19" s="4">
-        <f>(H19-G19)*L19*25</f>
-        <v/>
-      </c>
-      <c r="N19" s="4" t="n"/>
-      <c r="O19" s="4">
+      <c r="M19" s="4" t="n"/>
+      <c r="N19" s="4">
+        <f>(H19-G19)*L19*65</f>
+        <v/>
+      </c>
+      <c r="O19" s="4" t="n"/>
+      <c r="P19" s="4">
         <f>IFERROR((H19-G19)/(G19-I19),"—")</f>
         <v/>
       </c>
-      <c r="P19" s="4" t="n"/>
       <c r="Q19" s="4" t="n"/>
-      <c r="R19" s="5" t="n"/>
+      <c r="R19" s="4" t="n"/>
+      <c r="S19" s="5" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="6" t="n"/>
-      <c r="B20" s="6" t="n"/>
+      <c r="B20" s="39" t="n"/>
       <c r="C20" s="6" t="n"/>
       <c r="D20" s="6" t="n"/>
       <c r="E20" s="6" t="n"/>
@@ -1277,22 +1640,23 @@
       <c r="J20" s="6" t="n"/>
       <c r="K20" s="6" t="n"/>
       <c r="L20" s="6" t="n"/>
-      <c r="M20" s="6">
-        <f>(H20-G20)*L20*25</f>
-        <v/>
-      </c>
-      <c r="N20" s="6" t="n"/>
-      <c r="O20" s="6">
+      <c r="M20" s="6" t="n"/>
+      <c r="N20" s="6">
+        <f>(H20-G20)*L20*65</f>
+        <v/>
+      </c>
+      <c r="O20" s="6" t="n"/>
+      <c r="P20" s="6">
         <f>IFERROR((H20-G20)/(G20-I20),"—")</f>
         <v/>
       </c>
-      <c r="P20" s="6" t="n"/>
       <c r="Q20" s="6" t="n"/>
-      <c r="R20" s="7" t="n"/>
+      <c r="R20" s="6" t="n"/>
+      <c r="S20" s="7" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="4" t="n"/>
-      <c r="B21" s="4" t="n"/>
+      <c r="B21" s="39" t="n"/>
       <c r="C21" s="4" t="n"/>
       <c r="D21" s="4" t="n"/>
       <c r="E21" s="4" t="n"/>
@@ -1303,22 +1667,23 @@
       <c r="J21" s="4" t="n"/>
       <c r="K21" s="4" t="n"/>
       <c r="L21" s="4" t="n"/>
-      <c r="M21" s="4">
-        <f>(H21-G21)*L21*25</f>
-        <v/>
-      </c>
-      <c r="N21" s="4" t="n"/>
-      <c r="O21" s="4">
+      <c r="M21" s="4" t="n"/>
+      <c r="N21" s="4">
+        <f>(H21-G21)*L21*65</f>
+        <v/>
+      </c>
+      <c r="O21" s="4" t="n"/>
+      <c r="P21" s="4">
         <f>IFERROR((H21-G21)/(G21-I21),"—")</f>
         <v/>
       </c>
-      <c r="P21" s="4" t="n"/>
       <c r="Q21" s="4" t="n"/>
-      <c r="R21" s="5" t="n"/>
+      <c r="R21" s="4" t="n"/>
+      <c r="S21" s="5" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="n"/>
-      <c r="B22" s="6" t="n"/>
+      <c r="B22" s="39" t="n"/>
       <c r="C22" s="6" t="n"/>
       <c r="D22" s="6" t="n"/>
       <c r="E22" s="6" t="n"/>
@@ -1329,22 +1694,23 @@
       <c r="J22" s="6" t="n"/>
       <c r="K22" s="6" t="n"/>
       <c r="L22" s="6" t="n"/>
-      <c r="M22" s="6">
-        <f>(H22-G22)*L22*25</f>
-        <v/>
-      </c>
-      <c r="N22" s="6" t="n"/>
-      <c r="O22" s="6">
+      <c r="M22" s="6" t="n"/>
+      <c r="N22" s="6">
+        <f>(H22-G22)*L22*65</f>
+        <v/>
+      </c>
+      <c r="O22" s="6" t="n"/>
+      <c r="P22" s="6">
         <f>IFERROR((H22-G22)/(G22-I22),"—")</f>
         <v/>
       </c>
-      <c r="P22" s="6" t="n"/>
       <c r="Q22" s="6" t="n"/>
-      <c r="R22" s="7" t="n"/>
+      <c r="R22" s="6" t="n"/>
+      <c r="S22" s="7" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="4" t="n"/>
-      <c r="B23" s="4" t="n"/>
+      <c r="B23" s="39" t="n"/>
       <c r="C23" s="4" t="n"/>
       <c r="D23" s="4" t="n"/>
       <c r="E23" s="4" t="n"/>
@@ -1355,22 +1721,23 @@
       <c r="J23" s="4" t="n"/>
       <c r="K23" s="4" t="n"/>
       <c r="L23" s="4" t="n"/>
-      <c r="M23" s="4">
-        <f>(H23-G23)*L23*25</f>
-        <v/>
-      </c>
-      <c r="N23" s="4" t="n"/>
-      <c r="O23" s="4">
+      <c r="M23" s="4" t="n"/>
+      <c r="N23" s="4">
+        <f>(H23-G23)*L23*65</f>
+        <v/>
+      </c>
+      <c r="O23" s="4" t="n"/>
+      <c r="P23" s="4">
         <f>IFERROR((H23-G23)/(G23-I23),"—")</f>
         <v/>
       </c>
-      <c r="P23" s="4" t="n"/>
       <c r="Q23" s="4" t="n"/>
-      <c r="R23" s="5" t="n"/>
+      <c r="R23" s="4" t="n"/>
+      <c r="S23" s="5" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="6" t="n"/>
-      <c r="B24" s="6" t="n"/>
+      <c r="B24" s="39" t="n"/>
       <c r="C24" s="6" t="n"/>
       <c r="D24" s="6" t="n"/>
       <c r="E24" s="6" t="n"/>
@@ -1381,22 +1748,23 @@
       <c r="J24" s="6" t="n"/>
       <c r="K24" s="6" t="n"/>
       <c r="L24" s="6" t="n"/>
-      <c r="M24" s="6">
-        <f>(H24-G24)*L24*25</f>
-        <v/>
-      </c>
-      <c r="N24" s="6" t="n"/>
-      <c r="O24" s="6">
+      <c r="M24" s="6" t="n"/>
+      <c r="N24" s="6">
+        <f>(H24-G24)*L24*65</f>
+        <v/>
+      </c>
+      <c r="O24" s="6" t="n"/>
+      <c r="P24" s="6">
         <f>IFERROR((H24-G24)/(G24-I24),"—")</f>
         <v/>
       </c>
-      <c r="P24" s="6" t="n"/>
       <c r="Q24" s="6" t="n"/>
-      <c r="R24" s="7" t="n"/>
+      <c r="R24" s="6" t="n"/>
+      <c r="S24" s="7" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="4" t="n"/>
-      <c r="B25" s="4" t="n"/>
+      <c r="B25" s="39" t="n"/>
       <c r="C25" s="4" t="n"/>
       <c r="D25" s="4" t="n"/>
       <c r="E25" s="4" t="n"/>
@@ -1407,22 +1775,23 @@
       <c r="J25" s="4" t="n"/>
       <c r="K25" s="4" t="n"/>
       <c r="L25" s="4" t="n"/>
-      <c r="M25" s="4">
-        <f>(H25-G25)*L25*25</f>
-        <v/>
-      </c>
-      <c r="N25" s="4" t="n"/>
-      <c r="O25" s="4">
+      <c r="M25" s="4" t="n"/>
+      <c r="N25" s="4">
+        <f>(H25-G25)*L25*65</f>
+        <v/>
+      </c>
+      <c r="O25" s="4" t="n"/>
+      <c r="P25" s="4">
         <f>IFERROR((H25-G25)/(G25-I25),"—")</f>
         <v/>
       </c>
-      <c r="P25" s="4" t="n"/>
       <c r="Q25" s="4" t="n"/>
-      <c r="R25" s="5" t="n"/>
+      <c r="R25" s="4" t="n"/>
+      <c r="S25" s="5" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="6" t="n"/>
-      <c r="B26" s="6" t="n"/>
+      <c r="B26" s="39" t="n"/>
       <c r="C26" s="6" t="n"/>
       <c r="D26" s="6" t="n"/>
       <c r="E26" s="6" t="n"/>
@@ -1433,22 +1802,23 @@
       <c r="J26" s="6" t="n"/>
       <c r="K26" s="6" t="n"/>
       <c r="L26" s="6" t="n"/>
-      <c r="M26" s="6">
-        <f>(H26-G26)*L26*25</f>
-        <v/>
-      </c>
-      <c r="N26" s="6" t="n"/>
-      <c r="O26" s="6">
+      <c r="M26" s="6" t="n"/>
+      <c r="N26" s="6">
+        <f>(H26-G26)*L26*65</f>
+        <v/>
+      </c>
+      <c r="O26" s="6" t="n"/>
+      <c r="P26" s="6">
         <f>IFERROR((H26-G26)/(G26-I26),"—")</f>
         <v/>
       </c>
-      <c r="P26" s="6" t="n"/>
       <c r="Q26" s="6" t="n"/>
-      <c r="R26" s="7" t="n"/>
+      <c r="R26" s="6" t="n"/>
+      <c r="S26" s="7" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="4" t="n"/>
-      <c r="B27" s="4" t="n"/>
+      <c r="B27" s="39" t="n"/>
       <c r="C27" s="4" t="n"/>
       <c r="D27" s="4" t="n"/>
       <c r="E27" s="4" t="n"/>
@@ -1459,22 +1829,23 @@
       <c r="J27" s="4" t="n"/>
       <c r="K27" s="4" t="n"/>
       <c r="L27" s="4" t="n"/>
-      <c r="M27" s="4">
-        <f>(H27-G27)*L27*25</f>
-        <v/>
-      </c>
-      <c r="N27" s="4" t="n"/>
-      <c r="O27" s="4">
+      <c r="M27" s="4" t="n"/>
+      <c r="N27" s="4">
+        <f>(H27-G27)*L27*65</f>
+        <v/>
+      </c>
+      <c r="O27" s="4" t="n"/>
+      <c r="P27" s="4">
         <f>IFERROR((H27-G27)/(G27-I27),"—")</f>
         <v/>
       </c>
-      <c r="P27" s="4" t="n"/>
       <c r="Q27" s="4" t="n"/>
-      <c r="R27" s="5" t="n"/>
+      <c r="R27" s="4" t="n"/>
+      <c r="S27" s="5" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="6" t="n"/>
-      <c r="B28" s="6" t="n"/>
+      <c r="B28" s="39" t="n"/>
       <c r="C28" s="6" t="n"/>
       <c r="D28" s="6" t="n"/>
       <c r="E28" s="6" t="n"/>
@@ -1485,22 +1856,23 @@
       <c r="J28" s="6" t="n"/>
       <c r="K28" s="6" t="n"/>
       <c r="L28" s="6" t="n"/>
-      <c r="M28" s="6">
-        <f>(H28-G28)*L28*25</f>
-        <v/>
-      </c>
-      <c r="N28" s="6" t="n"/>
-      <c r="O28" s="6">
+      <c r="M28" s="6" t="n"/>
+      <c r="N28" s="6">
+        <f>(H28-G28)*L28*65</f>
+        <v/>
+      </c>
+      <c r="O28" s="6" t="n"/>
+      <c r="P28" s="6">
         <f>IFERROR((H28-G28)/(G28-I28),"—")</f>
         <v/>
       </c>
-      <c r="P28" s="6" t="n"/>
       <c r="Q28" s="6" t="n"/>
-      <c r="R28" s="7" t="n"/>
+      <c r="R28" s="6" t="n"/>
+      <c r="S28" s="7" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="4" t="n"/>
-      <c r="B29" s="4" t="n"/>
+      <c r="B29" s="39" t="n"/>
       <c r="C29" s="4" t="n"/>
       <c r="D29" s="4" t="n"/>
       <c r="E29" s="4" t="n"/>
@@ -1511,22 +1883,23 @@
       <c r="J29" s="4" t="n"/>
       <c r="K29" s="4" t="n"/>
       <c r="L29" s="4" t="n"/>
-      <c r="M29" s="4">
-        <f>(H29-G29)*L29*25</f>
-        <v/>
-      </c>
-      <c r="N29" s="4" t="n"/>
-      <c r="O29" s="4">
+      <c r="M29" s="4" t="n"/>
+      <c r="N29" s="4">
+        <f>(H29-G29)*L29*65</f>
+        <v/>
+      </c>
+      <c r="O29" s="4" t="n"/>
+      <c r="P29" s="4">
         <f>IFERROR((H29-G29)/(G29-I29),"—")</f>
         <v/>
       </c>
-      <c r="P29" s="4" t="n"/>
       <c r="Q29" s="4" t="n"/>
-      <c r="R29" s="5" t="n"/>
+      <c r="R29" s="4" t="n"/>
+      <c r="S29" s="5" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="6" t="n"/>
-      <c r="B30" s="6" t="n"/>
+      <c r="B30" s="39" t="n"/>
       <c r="C30" s="6" t="n"/>
       <c r="D30" s="6" t="n"/>
       <c r="E30" s="6" t="n"/>
@@ -1537,22 +1910,23 @@
       <c r="J30" s="6" t="n"/>
       <c r="K30" s="6" t="n"/>
       <c r="L30" s="6" t="n"/>
-      <c r="M30" s="6">
-        <f>(H30-G30)*L30*25</f>
-        <v/>
-      </c>
-      <c r="N30" s="6" t="n"/>
-      <c r="O30" s="6">
+      <c r="M30" s="6" t="n"/>
+      <c r="N30" s="6">
+        <f>(H30-G30)*L30*65</f>
+        <v/>
+      </c>
+      <c r="O30" s="6" t="n"/>
+      <c r="P30" s="6">
         <f>IFERROR((H30-G30)/(G30-I30),"—")</f>
         <v/>
       </c>
-      <c r="P30" s="6" t="n"/>
       <c r="Q30" s="6" t="n"/>
-      <c r="R30" s="7" t="n"/>
+      <c r="R30" s="6" t="n"/>
+      <c r="S30" s="7" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="4" t="n"/>
-      <c r="B31" s="4" t="n"/>
+      <c r="B31" s="39" t="n"/>
       <c r="C31" s="4" t="n"/>
       <c r="D31" s="4" t="n"/>
       <c r="E31" s="4" t="n"/>
@@ -1563,22 +1937,23 @@
       <c r="J31" s="4" t="n"/>
       <c r="K31" s="4" t="n"/>
       <c r="L31" s="4" t="n"/>
-      <c r="M31" s="4">
-        <f>(H31-G31)*L31*25</f>
-        <v/>
-      </c>
-      <c r="N31" s="4" t="n"/>
-      <c r="O31" s="4">
+      <c r="M31" s="4" t="n"/>
+      <c r="N31" s="4">
+        <f>(H31-G31)*L31*65</f>
+        <v/>
+      </c>
+      <c r="O31" s="4" t="n"/>
+      <c r="P31" s="4">
         <f>IFERROR((H31-G31)/(G31-I31),"—")</f>
         <v/>
       </c>
-      <c r="P31" s="4" t="n"/>
       <c r="Q31" s="4" t="n"/>
-      <c r="R31" s="5" t="n"/>
+      <c r="R31" s="4" t="n"/>
+      <c r="S31" s="5" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="6" t="n"/>
-      <c r="B32" s="6" t="n"/>
+      <c r="B32" s="39" t="n"/>
       <c r="C32" s="6" t="n"/>
       <c r="D32" s="6" t="n"/>
       <c r="E32" s="6" t="n"/>
@@ -1589,22 +1964,23 @@
       <c r="J32" s="6" t="n"/>
       <c r="K32" s="6" t="n"/>
       <c r="L32" s="6" t="n"/>
-      <c r="M32" s="6">
-        <f>(H32-G32)*L32*25</f>
-        <v/>
-      </c>
-      <c r="N32" s="6" t="n"/>
-      <c r="O32" s="6">
+      <c r="M32" s="6" t="n"/>
+      <c r="N32" s="6">
+        <f>(H32-G32)*L32*65</f>
+        <v/>
+      </c>
+      <c r="O32" s="6" t="n"/>
+      <c r="P32" s="6">
         <f>IFERROR((H32-G32)/(G32-I32),"—")</f>
         <v/>
       </c>
-      <c r="P32" s="6" t="n"/>
       <c r="Q32" s="6" t="n"/>
-      <c r="R32" s="7" t="n"/>
+      <c r="R32" s="6" t="n"/>
+      <c r="S32" s="7" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="4" t="n"/>
-      <c r="B33" s="4" t="n"/>
+      <c r="B33" s="39" t="n"/>
       <c r="C33" s="4" t="n"/>
       <c r="D33" s="4" t="n"/>
       <c r="E33" s="4" t="n"/>
@@ -1615,22 +1991,23 @@
       <c r="J33" s="4" t="n"/>
       <c r="K33" s="4" t="n"/>
       <c r="L33" s="4" t="n"/>
-      <c r="M33" s="4">
-        <f>(H33-G33)*L33*25</f>
-        <v/>
-      </c>
-      <c r="N33" s="4" t="n"/>
-      <c r="O33" s="4">
+      <c r="M33" s="4" t="n"/>
+      <c r="N33" s="4">
+        <f>(H33-G33)*L33*65</f>
+        <v/>
+      </c>
+      <c r="O33" s="4" t="n"/>
+      <c r="P33" s="4">
         <f>IFERROR((H33-G33)/(G33-I33),"—")</f>
         <v/>
       </c>
-      <c r="P33" s="4" t="n"/>
       <c r="Q33" s="4" t="n"/>
-      <c r="R33" s="5" t="n"/>
+      <c r="R33" s="4" t="n"/>
+      <c r="S33" s="5" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="6" t="n"/>
-      <c r="B34" s="6" t="n"/>
+      <c r="B34" s="39" t="n"/>
       <c r="C34" s="6" t="n"/>
       <c r="D34" s="6" t="n"/>
       <c r="E34" s="6" t="n"/>
@@ -1641,22 +2018,23 @@
       <c r="J34" s="6" t="n"/>
       <c r="K34" s="6" t="n"/>
       <c r="L34" s="6" t="n"/>
-      <c r="M34" s="6">
-        <f>(H34-G34)*L34*25</f>
-        <v/>
-      </c>
-      <c r="N34" s="6" t="n"/>
-      <c r="O34" s="6">
+      <c r="M34" s="6" t="n"/>
+      <c r="N34" s="6">
+        <f>(H34-G34)*L34*65</f>
+        <v/>
+      </c>
+      <c r="O34" s="6" t="n"/>
+      <c r="P34" s="6">
         <f>IFERROR((H34-G34)/(G34-I34),"—")</f>
         <v/>
       </c>
-      <c r="P34" s="6" t="n"/>
       <c r="Q34" s="6" t="n"/>
-      <c r="R34" s="7" t="n"/>
+      <c r="R34" s="6" t="n"/>
+      <c r="S34" s="7" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="4" t="n"/>
-      <c r="B35" s="4" t="n"/>
+      <c r="B35" s="39" t="n"/>
       <c r="C35" s="4" t="n"/>
       <c r="D35" s="4" t="n"/>
       <c r="E35" s="4" t="n"/>
@@ -1667,22 +2045,23 @@
       <c r="J35" s="4" t="n"/>
       <c r="K35" s="4" t="n"/>
       <c r="L35" s="4" t="n"/>
-      <c r="M35" s="4">
-        <f>(H35-G35)*L35*25</f>
-        <v/>
-      </c>
-      <c r="N35" s="4" t="n"/>
-      <c r="O35" s="4">
+      <c r="M35" s="4" t="n"/>
+      <c r="N35" s="4">
+        <f>(H35-G35)*L35*65</f>
+        <v/>
+      </c>
+      <c r="O35" s="4" t="n"/>
+      <c r="P35" s="4">
         <f>IFERROR((H35-G35)/(G35-I35),"—")</f>
         <v/>
       </c>
-      <c r="P35" s="4" t="n"/>
       <c r="Q35" s="4" t="n"/>
-      <c r="R35" s="5" t="n"/>
+      <c r="R35" s="4" t="n"/>
+      <c r="S35" s="5" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="6" t="n"/>
-      <c r="B36" s="6" t="n"/>
+      <c r="B36" s="39" t="n"/>
       <c r="C36" s="6" t="n"/>
       <c r="D36" s="6" t="n"/>
       <c r="E36" s="6" t="n"/>
@@ -1693,22 +2072,23 @@
       <c r="J36" s="6" t="n"/>
       <c r="K36" s="6" t="n"/>
       <c r="L36" s="6" t="n"/>
-      <c r="M36" s="6">
-        <f>(H36-G36)*L36*25</f>
-        <v/>
-      </c>
-      <c r="N36" s="6" t="n"/>
-      <c r="O36" s="6">
+      <c r="M36" s="6" t="n"/>
+      <c r="N36" s="6">
+        <f>(H36-G36)*L36*65</f>
+        <v/>
+      </c>
+      <c r="O36" s="6" t="n"/>
+      <c r="P36" s="6">
         <f>IFERROR((H36-G36)/(G36-I36),"—")</f>
         <v/>
       </c>
-      <c r="P36" s="6" t="n"/>
       <c r="Q36" s="6" t="n"/>
-      <c r="R36" s="7" t="n"/>
+      <c r="R36" s="6" t="n"/>
+      <c r="S36" s="7" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="4" t="n"/>
-      <c r="B37" s="4" t="n"/>
+      <c r="B37" s="39" t="n"/>
       <c r="C37" s="4" t="n"/>
       <c r="D37" s="4" t="n"/>
       <c r="E37" s="4" t="n"/>
@@ -1719,22 +2099,23 @@
       <c r="J37" s="4" t="n"/>
       <c r="K37" s="4" t="n"/>
       <c r="L37" s="4" t="n"/>
-      <c r="M37" s="4">
-        <f>(H37-G37)*L37*25</f>
-        <v/>
-      </c>
-      <c r="N37" s="4" t="n"/>
-      <c r="O37" s="4">
+      <c r="M37" s="4" t="n"/>
+      <c r="N37" s="4">
+        <f>(H37-G37)*L37*65</f>
+        <v/>
+      </c>
+      <c r="O37" s="4" t="n"/>
+      <c r="P37" s="4">
         <f>IFERROR((H37-G37)/(G37-I37),"—")</f>
         <v/>
       </c>
-      <c r="P37" s="4" t="n"/>
       <c r="Q37" s="4" t="n"/>
-      <c r="R37" s="5" t="n"/>
+      <c r="R37" s="4" t="n"/>
+      <c r="S37" s="5" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="6" t="n"/>
-      <c r="B38" s="6" t="n"/>
+      <c r="B38" s="39" t="n"/>
       <c r="C38" s="6" t="n"/>
       <c r="D38" s="6" t="n"/>
       <c r="E38" s="6" t="n"/>
@@ -1745,22 +2126,23 @@
       <c r="J38" s="6" t="n"/>
       <c r="K38" s="6" t="n"/>
       <c r="L38" s="6" t="n"/>
-      <c r="M38" s="6">
-        <f>(H38-G38)*L38*25</f>
-        <v/>
-      </c>
-      <c r="N38" s="6" t="n"/>
-      <c r="O38" s="6">
+      <c r="M38" s="6" t="n"/>
+      <c r="N38" s="6">
+        <f>(H38-G38)*L38*65</f>
+        <v/>
+      </c>
+      <c r="O38" s="6" t="n"/>
+      <c r="P38" s="6">
         <f>IFERROR((H38-G38)/(G38-I38),"—")</f>
         <v/>
       </c>
-      <c r="P38" s="6" t="n"/>
       <c r="Q38" s="6" t="n"/>
-      <c r="R38" s="7" t="n"/>
+      <c r="R38" s="6" t="n"/>
+      <c r="S38" s="7" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="4" t="n"/>
-      <c r="B39" s="4" t="n"/>
+      <c r="B39" s="39" t="n"/>
       <c r="C39" s="4" t="n"/>
       <c r="D39" s="4" t="n"/>
       <c r="E39" s="4" t="n"/>
@@ -1771,22 +2153,23 @@
       <c r="J39" s="4" t="n"/>
       <c r="K39" s="4" t="n"/>
       <c r="L39" s="4" t="n"/>
-      <c r="M39" s="4">
-        <f>(H39-G39)*L39*25</f>
-        <v/>
-      </c>
-      <c r="N39" s="4" t="n"/>
-      <c r="O39" s="4">
+      <c r="M39" s="4" t="n"/>
+      <c r="N39" s="4">
+        <f>(H39-G39)*L39*65</f>
+        <v/>
+      </c>
+      <c r="O39" s="4" t="n"/>
+      <c r="P39" s="4">
         <f>IFERROR((H39-G39)/(G39-I39),"—")</f>
         <v/>
       </c>
-      <c r="P39" s="4" t="n"/>
       <c r="Q39" s="4" t="n"/>
-      <c r="R39" s="5" t="n"/>
+      <c r="R39" s="4" t="n"/>
+      <c r="S39" s="5" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="6" t="n"/>
-      <c r="B40" s="6" t="n"/>
+      <c r="B40" s="39" t="n"/>
       <c r="C40" s="6" t="n"/>
       <c r="D40" s="6" t="n"/>
       <c r="E40" s="6" t="n"/>
@@ -1797,22 +2180,23 @@
       <c r="J40" s="6" t="n"/>
       <c r="K40" s="6" t="n"/>
       <c r="L40" s="6" t="n"/>
-      <c r="M40" s="6">
-        <f>(H40-G40)*L40*25</f>
-        <v/>
-      </c>
-      <c r="N40" s="6" t="n"/>
-      <c r="O40" s="6">
+      <c r="M40" s="6" t="n"/>
+      <c r="N40" s="6">
+        <f>(H40-G40)*L40*65</f>
+        <v/>
+      </c>
+      <c r="O40" s="6" t="n"/>
+      <c r="P40" s="6">
         <f>IFERROR((H40-G40)/(G40-I40),"—")</f>
         <v/>
       </c>
-      <c r="P40" s="6" t="n"/>
       <c r="Q40" s="6" t="n"/>
-      <c r="R40" s="7" t="n"/>
+      <c r="R40" s="6" t="n"/>
+      <c r="S40" s="7" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="4" t="n"/>
-      <c r="B41" s="4" t="n"/>
+      <c r="B41" s="39" t="n"/>
       <c r="C41" s="4" t="n"/>
       <c r="D41" s="4" t="n"/>
       <c r="E41" s="4" t="n"/>
@@ -1823,22 +2207,23 @@
       <c r="J41" s="4" t="n"/>
       <c r="K41" s="4" t="n"/>
       <c r="L41" s="4" t="n"/>
-      <c r="M41" s="4">
-        <f>(H41-G41)*L41*25</f>
-        <v/>
-      </c>
-      <c r="N41" s="4" t="n"/>
-      <c r="O41" s="4">
+      <c r="M41" s="4" t="n"/>
+      <c r="N41" s="4">
+        <f>(H41-G41)*L41*65</f>
+        <v/>
+      </c>
+      <c r="O41" s="4" t="n"/>
+      <c r="P41" s="4">
         <f>IFERROR((H41-G41)/(G41-I41),"—")</f>
         <v/>
       </c>
-      <c r="P41" s="4" t="n"/>
       <c r="Q41" s="4" t="n"/>
-      <c r="R41" s="5" t="n"/>
+      <c r="R41" s="4" t="n"/>
+      <c r="S41" s="5" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="6" t="n"/>
-      <c r="B42" s="6" t="n"/>
+      <c r="B42" s="39" t="n"/>
       <c r="C42" s="6" t="n"/>
       <c r="D42" s="6" t="n"/>
       <c r="E42" s="6" t="n"/>
@@ -1849,22 +2234,23 @@
       <c r="J42" s="6" t="n"/>
       <c r="K42" s="6" t="n"/>
       <c r="L42" s="6" t="n"/>
-      <c r="M42" s="6">
-        <f>(H42-G42)*L42*25</f>
-        <v/>
-      </c>
-      <c r="N42" s="6" t="n"/>
-      <c r="O42" s="6">
+      <c r="M42" s="6" t="n"/>
+      <c r="N42" s="6">
+        <f>(H42-G42)*L42*65</f>
+        <v/>
+      </c>
+      <c r="O42" s="6" t="n"/>
+      <c r="P42" s="6">
         <f>IFERROR((H42-G42)/(G42-I42),"—")</f>
         <v/>
       </c>
-      <c r="P42" s="6" t="n"/>
       <c r="Q42" s="6" t="n"/>
-      <c r="R42" s="7" t="n"/>
+      <c r="R42" s="6" t="n"/>
+      <c r="S42" s="7" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="4" t="n"/>
-      <c r="B43" s="4" t="n"/>
+      <c r="B43" s="39" t="n"/>
       <c r="C43" s="4" t="n"/>
       <c r="D43" s="4" t="n"/>
       <c r="E43" s="4" t="n"/>
@@ -1875,22 +2261,23 @@
       <c r="J43" s="4" t="n"/>
       <c r="K43" s="4" t="n"/>
       <c r="L43" s="4" t="n"/>
-      <c r="M43" s="4">
-        <f>(H43-G43)*L43*25</f>
-        <v/>
-      </c>
-      <c r="N43" s="4" t="n"/>
-      <c r="O43" s="4">
+      <c r="M43" s="4" t="n"/>
+      <c r="N43" s="4">
+        <f>(H43-G43)*L43*65</f>
+        <v/>
+      </c>
+      <c r="O43" s="4" t="n"/>
+      <c r="P43" s="4">
         <f>IFERROR((H43-G43)/(G43-I43),"—")</f>
         <v/>
       </c>
-      <c r="P43" s="4" t="n"/>
       <c r="Q43" s="4" t="n"/>
-      <c r="R43" s="5" t="n"/>
+      <c r="R43" s="4" t="n"/>
+      <c r="S43" s="5" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="6" t="n"/>
-      <c r="B44" s="6" t="n"/>
+      <c r="B44" s="39" t="n"/>
       <c r="C44" s="6" t="n"/>
       <c r="D44" s="6" t="n"/>
       <c r="E44" s="6" t="n"/>
@@ -1901,22 +2288,23 @@
       <c r="J44" s="6" t="n"/>
       <c r="K44" s="6" t="n"/>
       <c r="L44" s="6" t="n"/>
-      <c r="M44" s="6">
-        <f>(H44-G44)*L44*25</f>
-        <v/>
-      </c>
-      <c r="N44" s="6" t="n"/>
-      <c r="O44" s="6">
+      <c r="M44" s="6" t="n"/>
+      <c r="N44" s="6">
+        <f>(H44-G44)*L44*65</f>
+        <v/>
+      </c>
+      <c r="O44" s="6" t="n"/>
+      <c r="P44" s="6">
         <f>IFERROR((H44-G44)/(G44-I44),"—")</f>
         <v/>
       </c>
-      <c r="P44" s="6" t="n"/>
       <c r="Q44" s="6" t="n"/>
-      <c r="R44" s="7" t="n"/>
+      <c r="R44" s="6" t="n"/>
+      <c r="S44" s="7" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="4" t="n"/>
-      <c r="B45" s="4" t="n"/>
+      <c r="B45" s="39" t="n"/>
       <c r="C45" s="4" t="n"/>
       <c r="D45" s="4" t="n"/>
       <c r="E45" s="4" t="n"/>
@@ -1927,22 +2315,23 @@
       <c r="J45" s="4" t="n"/>
       <c r="K45" s="4" t="n"/>
       <c r="L45" s="4" t="n"/>
-      <c r="M45" s="4">
-        <f>(H45-G45)*L45*25</f>
-        <v/>
-      </c>
-      <c r="N45" s="4" t="n"/>
-      <c r="O45" s="4">
+      <c r="M45" s="4" t="n"/>
+      <c r="N45" s="4">
+        <f>(H45-G45)*L45*65</f>
+        <v/>
+      </c>
+      <c r="O45" s="4" t="n"/>
+      <c r="P45" s="4">
         <f>IFERROR((H45-G45)/(G45-I45),"—")</f>
         <v/>
       </c>
-      <c r="P45" s="4" t="n"/>
       <c r="Q45" s="4" t="n"/>
-      <c r="R45" s="5" t="n"/>
+      <c r="R45" s="4" t="n"/>
+      <c r="S45" s="5" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="6" t="n"/>
-      <c r="B46" s="6" t="n"/>
+      <c r="B46" s="39" t="n"/>
       <c r="C46" s="6" t="n"/>
       <c r="D46" s="6" t="n"/>
       <c r="E46" s="6" t="n"/>
@@ -1953,22 +2342,23 @@
       <c r="J46" s="6" t="n"/>
       <c r="K46" s="6" t="n"/>
       <c r="L46" s="6" t="n"/>
-      <c r="M46" s="6">
-        <f>(H46-G46)*L46*25</f>
-        <v/>
-      </c>
-      <c r="N46" s="6" t="n"/>
-      <c r="O46" s="6">
+      <c r="M46" s="6" t="n"/>
+      <c r="N46" s="6">
+        <f>(H46-G46)*L46*65</f>
+        <v/>
+      </c>
+      <c r="O46" s="6" t="n"/>
+      <c r="P46" s="6">
         <f>IFERROR((H46-G46)/(G46-I46),"—")</f>
         <v/>
       </c>
-      <c r="P46" s="6" t="n"/>
       <c r="Q46" s="6" t="n"/>
-      <c r="R46" s="7" t="n"/>
+      <c r="R46" s="6" t="n"/>
+      <c r="S46" s="7" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="4" t="n"/>
-      <c r="B47" s="4" t="n"/>
+      <c r="B47" s="39" t="n"/>
       <c r="C47" s="4" t="n"/>
       <c r="D47" s="4" t="n"/>
       <c r="E47" s="4" t="n"/>
@@ -1979,22 +2369,23 @@
       <c r="J47" s="4" t="n"/>
       <c r="K47" s="4" t="n"/>
       <c r="L47" s="4" t="n"/>
-      <c r="M47" s="4">
-        <f>(H47-G47)*L47*25</f>
-        <v/>
-      </c>
-      <c r="N47" s="4" t="n"/>
-      <c r="O47" s="4">
+      <c r="M47" s="4" t="n"/>
+      <c r="N47" s="4">
+        <f>(H47-G47)*L47*65</f>
+        <v/>
+      </c>
+      <c r="O47" s="4" t="n"/>
+      <c r="P47" s="4">
         <f>IFERROR((H47-G47)/(G47-I47),"—")</f>
         <v/>
       </c>
-      <c r="P47" s="4" t="n"/>
       <c r="Q47" s="4" t="n"/>
-      <c r="R47" s="5" t="n"/>
+      <c r="R47" s="4" t="n"/>
+      <c r="S47" s="5" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="6" t="n"/>
-      <c r="B48" s="6" t="n"/>
+      <c r="B48" s="39" t="n"/>
       <c r="C48" s="6" t="n"/>
       <c r="D48" s="6" t="n"/>
       <c r="E48" s="6" t="n"/>
@@ -2005,22 +2396,23 @@
       <c r="J48" s="6" t="n"/>
       <c r="K48" s="6" t="n"/>
       <c r="L48" s="6" t="n"/>
-      <c r="M48" s="6">
-        <f>(H48-G48)*L48*25</f>
-        <v/>
-      </c>
-      <c r="N48" s="6" t="n"/>
-      <c r="O48" s="6">
+      <c r="M48" s="6" t="n"/>
+      <c r="N48" s="6">
+        <f>(H48-G48)*L48*65</f>
+        <v/>
+      </c>
+      <c r="O48" s="6" t="n"/>
+      <c r="P48" s="6">
         <f>IFERROR((H48-G48)/(G48-I48),"—")</f>
         <v/>
       </c>
-      <c r="P48" s="6" t="n"/>
       <c r="Q48" s="6" t="n"/>
-      <c r="R48" s="7" t="n"/>
+      <c r="R48" s="6" t="n"/>
+      <c r="S48" s="7" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="4" t="n"/>
-      <c r="B49" s="4" t="n"/>
+      <c r="B49" s="39" t="n"/>
       <c r="C49" s="4" t="n"/>
       <c r="D49" s="4" t="n"/>
       <c r="E49" s="4" t="n"/>
@@ -2031,22 +2423,23 @@
       <c r="J49" s="4" t="n"/>
       <c r="K49" s="4" t="n"/>
       <c r="L49" s="4" t="n"/>
-      <c r="M49" s="4">
-        <f>(H49-G49)*L49*25</f>
-        <v/>
-      </c>
-      <c r="N49" s="4" t="n"/>
-      <c r="O49" s="4">
+      <c r="M49" s="4" t="n"/>
+      <c r="N49" s="4">
+        <f>(H49-G49)*L49*65</f>
+        <v/>
+      </c>
+      <c r="O49" s="4" t="n"/>
+      <c r="P49" s="4">
         <f>IFERROR((H49-G49)/(G49-I49),"—")</f>
         <v/>
       </c>
-      <c r="P49" s="4" t="n"/>
       <c r="Q49" s="4" t="n"/>
-      <c r="R49" s="5" t="n"/>
+      <c r="R49" s="4" t="n"/>
+      <c r="S49" s="5" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="6" t="n"/>
-      <c r="B50" s="6" t="n"/>
+      <c r="B50" s="39" t="n"/>
       <c r="C50" s="6" t="n"/>
       <c r="D50" s="6" t="n"/>
       <c r="E50" s="6" t="n"/>
@@ -2057,22 +2450,23 @@
       <c r="J50" s="6" t="n"/>
       <c r="K50" s="6" t="n"/>
       <c r="L50" s="6" t="n"/>
-      <c r="M50" s="6">
-        <f>(H50-G50)*L50*25</f>
-        <v/>
-      </c>
-      <c r="N50" s="6" t="n"/>
-      <c r="O50" s="6">
+      <c r="M50" s="6" t="n"/>
+      <c r="N50" s="6">
+        <f>(H50-G50)*L50*65</f>
+        <v/>
+      </c>
+      <c r="O50" s="6" t="n"/>
+      <c r="P50" s="6">
         <f>IFERROR((H50-G50)/(G50-I50),"—")</f>
         <v/>
       </c>
-      <c r="P50" s="6" t="n"/>
       <c r="Q50" s="6" t="n"/>
-      <c r="R50" s="7" t="n"/>
+      <c r="R50" s="6" t="n"/>
+      <c r="S50" s="7" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="4" t="n"/>
-      <c r="B51" s="4" t="n"/>
+      <c r="B51" s="39" t="n"/>
       <c r="C51" s="4" t="n"/>
       <c r="D51" s="4" t="n"/>
       <c r="E51" s="4" t="n"/>
@@ -2083,22 +2477,23 @@
       <c r="J51" s="4" t="n"/>
       <c r="K51" s="4" t="n"/>
       <c r="L51" s="4" t="n"/>
-      <c r="M51" s="4">
-        <f>(H51-G51)*L51*25</f>
-        <v/>
-      </c>
-      <c r="N51" s="4" t="n"/>
-      <c r="O51" s="4">
+      <c r="M51" s="4" t="n"/>
+      <c r="N51" s="4">
+        <f>(H51-G51)*L51*65</f>
+        <v/>
+      </c>
+      <c r="O51" s="4" t="n"/>
+      <c r="P51" s="4">
         <f>IFERROR((H51-G51)/(G51-I51),"—")</f>
         <v/>
       </c>
-      <c r="P51" s="4" t="n"/>
       <c r="Q51" s="4" t="n"/>
-      <c r="R51" s="5" t="n"/>
+      <c r="R51" s="4" t="n"/>
+      <c r="S51" s="5" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="6" t="n"/>
-      <c r="B52" s="6" t="n"/>
+      <c r="B52" s="39" t="n"/>
       <c r="C52" s="6" t="n"/>
       <c r="D52" s="6" t="n"/>
       <c r="E52" s="6" t="n"/>
@@ -2109,22 +2504,23 @@
       <c r="J52" s="6" t="n"/>
       <c r="K52" s="6" t="n"/>
       <c r="L52" s="6" t="n"/>
-      <c r="M52" s="6">
-        <f>(H52-G52)*L52*25</f>
-        <v/>
-      </c>
-      <c r="N52" s="6" t="n"/>
-      <c r="O52" s="6">
+      <c r="M52" s="6" t="n"/>
+      <c r="N52" s="6">
+        <f>(H52-G52)*L52*65</f>
+        <v/>
+      </c>
+      <c r="O52" s="6" t="n"/>
+      <c r="P52" s="6">
         <f>IFERROR((H52-G52)/(G52-I52),"—")</f>
         <v/>
       </c>
-      <c r="P52" s="6" t="n"/>
       <c r="Q52" s="6" t="n"/>
-      <c r="R52" s="7" t="n"/>
+      <c r="R52" s="6" t="n"/>
+      <c r="S52" s="7" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="4" t="n"/>
-      <c r="B53" s="4" t="n"/>
+      <c r="B53" s="39" t="n"/>
       <c r="C53" s="4" t="n"/>
       <c r="D53" s="4" t="n"/>
       <c r="E53" s="4" t="n"/>
@@ -2135,22 +2531,23 @@
       <c r="J53" s="4" t="n"/>
       <c r="K53" s="4" t="n"/>
       <c r="L53" s="4" t="n"/>
-      <c r="M53" s="4">
-        <f>(H53-G53)*L53*25</f>
-        <v/>
-      </c>
-      <c r="N53" s="4" t="n"/>
-      <c r="O53" s="4">
+      <c r="M53" s="4" t="n"/>
+      <c r="N53" s="4">
+        <f>(H53-G53)*L53*65</f>
+        <v/>
+      </c>
+      <c r="O53" s="4" t="n"/>
+      <c r="P53" s="4">
         <f>IFERROR((H53-G53)/(G53-I53),"—")</f>
         <v/>
       </c>
-      <c r="P53" s="4" t="n"/>
       <c r="Q53" s="4" t="n"/>
-      <c r="R53" s="5" t="n"/>
+      <c r="R53" s="4" t="n"/>
+      <c r="S53" s="5" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="6" t="n"/>
-      <c r="B54" s="6" t="n"/>
+      <c r="B54" s="39" t="n"/>
       <c r="C54" s="6" t="n"/>
       <c r="D54" s="6" t="n"/>
       <c r="E54" s="6" t="n"/>
@@ -2161,18 +2558,19 @@
       <c r="J54" s="6" t="n"/>
       <c r="K54" s="6" t="n"/>
       <c r="L54" s="6" t="n"/>
-      <c r="M54" s="6">
-        <f>(H54-G54)*L54*25</f>
-        <v/>
-      </c>
-      <c r="N54" s="6" t="n"/>
-      <c r="O54" s="6">
+      <c r="M54" s="6" t="n"/>
+      <c r="N54" s="6">
+        <f>(H54-G54)*L54*65</f>
+        <v/>
+      </c>
+      <c r="O54" s="6" t="n"/>
+      <c r="P54" s="6">
         <f>IFERROR((H54-G54)/(G54-I54),"—")</f>
         <v/>
       </c>
-      <c r="P54" s="6" t="n"/>
       <c r="Q54" s="6" t="n"/>
-      <c r="R54" s="7" t="n"/>
+      <c r="R54" s="6" t="n"/>
+      <c r="S54" s="7" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -2202,7 +2600,7 @@
       </colorScale>
     </cfRule>
   </conditionalFormatting>
-  <dataValidations count="5">
+  <dataValidations count="6">
     <dataValidation sqref="E5:E54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"PE Buy,CE Buy,Put Sell,Call Sell"</formula1>
     </dataValidation>
@@ -2218,6 +2616,9 @@
     <dataValidation sqref="B5:B54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"Mon,Tue,Wed,Thu,Fri"</formula1>
     </dataValidation>
+    <dataValidation sqref="B5:B54" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+      <formula1>"Intraday,Swing"</formula1>
+    </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2229,7 +2630,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J23"/>
+  <dimension ref="A1:J31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -2286,7 +2687,7 @@
         </is>
       </c>
       <c r="B5" s="10">
-        <f>COUNTIF('Trade Journal'!N5:N54,"Profit")</f>
+        <f>COUNTIF('Trade Journal'!O5:O54,"Profit")</f>
         <v/>
       </c>
       <c r="F5" s="12" t="inlineStr">
@@ -2322,7 +2723,7 @@
         </is>
       </c>
       <c r="B6" s="10">
-        <f>COUNTIF('Trade Journal'!N5:N54,"Loss")</f>
+        <f>COUNTIF('Trade Journal'!O5:O54,"Loss")</f>
         <v/>
       </c>
       <c r="F6" s="4" t="inlineStr">
@@ -2331,15 +2732,15 @@
         </is>
       </c>
       <c r="G6" s="4">
-        <f>COUNTIF('Trade Journal'!E5:E54,"PE Buy")</f>
+        <f>COUNTIF('Trade Journal'!F5:F54,"PE Buy")</f>
         <v/>
       </c>
       <c r="H6" s="4">
-        <f>COUNTIFS('Trade Journal'!E5:E54,"PE Buy",'Trade Journal'!N5:N54,"Profit")</f>
+        <f>COUNTIFS('Trade Journal'!F5:F54,"PE Buy",'Trade Journal'!O5:O54,"Profit")</f>
         <v/>
       </c>
       <c r="I6" s="4">
-        <f>COUNTIFS('Trade Journal'!E5:E54,"PE Buy",'Trade Journal'!N5:N54,"Loss")</f>
+        <f>COUNTIFS('Trade Journal'!F5:F54,"PE Buy",'Trade Journal'!O5:O54,"Loss")</f>
         <v/>
       </c>
       <c r="J6" s="13">
@@ -2354,7 +2755,7 @@
         </is>
       </c>
       <c r="B7" s="10">
-        <f>COUNTIF('Trade Journal'!N5:N54,"Breakeven")</f>
+        <f>COUNTIF('Trade Journal'!O5:O54,"Breakeven")</f>
         <v/>
       </c>
       <c r="F7" s="6" t="inlineStr">
@@ -2363,15 +2764,15 @@
         </is>
       </c>
       <c r="G7" s="6">
-        <f>COUNTIF('Trade Journal'!E5:E54,"CE Buy")</f>
+        <f>COUNTIF('Trade Journal'!F5:F54,"CE Buy")</f>
         <v/>
       </c>
       <c r="H7" s="6">
-        <f>COUNTIFS('Trade Journal'!E5:E54,"CE Buy",'Trade Journal'!N5:N54,"Profit")</f>
+        <f>COUNTIFS('Trade Journal'!F5:F54,"CE Buy",'Trade Journal'!O5:O54,"Profit")</f>
         <v/>
       </c>
       <c r="I7" s="6">
-        <f>COUNTIFS('Trade Journal'!E5:E54,"CE Buy",'Trade Journal'!N5:N54,"Loss")</f>
+        <f>COUNTIFS('Trade Journal'!F5:F54,"CE Buy",'Trade Journal'!O5:O54,"Loss")</f>
         <v/>
       </c>
       <c r="J7" s="14">
@@ -2395,15 +2796,15 @@
         </is>
       </c>
       <c r="G8" s="4">
-        <f>COUNTIF('Trade Journal'!E5:E54,"Put Sell")</f>
+        <f>COUNTIF('Trade Journal'!F5:F54,"Put Sell")</f>
         <v/>
       </c>
       <c r="H8" s="4">
-        <f>COUNTIFS('Trade Journal'!E5:E54,"Put Sell",'Trade Journal'!N5:N54,"Profit")</f>
+        <f>COUNTIFS('Trade Journal'!F5:F54,"Put Sell",'Trade Journal'!O5:O54,"Profit")</f>
         <v/>
       </c>
       <c r="I8" s="4">
-        <f>COUNTIFS('Trade Journal'!E5:E54,"Put Sell",'Trade Journal'!N5:N54,"Loss")</f>
+        <f>COUNTIFS('Trade Journal'!F5:F54,"Put Sell",'Trade Journal'!O5:O54,"Loss")</f>
         <v/>
       </c>
       <c r="J8" s="13">
@@ -2418,7 +2819,7 @@
         </is>
       </c>
       <c r="B9" s="16">
-        <f>SUM('Trade Journal'!M5:M54)</f>
+        <f>SUM('Trade Journal'!N5:N54)</f>
         <v/>
       </c>
       <c r="F9" s="6" t="inlineStr">
@@ -2427,15 +2828,15 @@
         </is>
       </c>
       <c r="G9" s="6">
-        <f>COUNTIF('Trade Journal'!E5:E54,"Call Sell")</f>
+        <f>COUNTIF('Trade Journal'!F5:F54,"Call Sell")</f>
         <v/>
       </c>
       <c r="H9" s="6">
-        <f>COUNTIFS('Trade Journal'!E5:E54,"Call Sell",'Trade Journal'!N5:N54,"Profit")</f>
+        <f>COUNTIFS('Trade Journal'!F5:F54,"Call Sell",'Trade Journal'!O5:O54,"Profit")</f>
         <v/>
       </c>
       <c r="I9" s="6">
-        <f>COUNTIFS('Trade Journal'!E5:E54,"Call Sell",'Trade Journal'!N5:N54,"Loss")</f>
+        <f>COUNTIFS('Trade Journal'!F5:F54,"Call Sell",'Trade Journal'!O5:O54,"Loss")</f>
         <v/>
       </c>
       <c r="J9" s="14">
@@ -2450,7 +2851,7 @@
         </is>
       </c>
       <c r="B10" s="16">
-        <f>IFERROR(AVERAGEIF('Trade Journal'!N5:N54,"Profit",'Trade Journal'!M5:M54),0)</f>
+        <f>IFERROR(AVERAGEIF('Trade Journal'!O5:O54,"Profit",'Trade Journal'!N5:N54),0)</f>
         <v/>
       </c>
     </row>
@@ -2461,7 +2862,7 @@
         </is>
       </c>
       <c r="B11" s="16">
-        <f>IFERROR(AVERAGEIF('Trade Journal'!N5:N54,"Loss",'Trade Journal'!M5:M54),0)</f>
+        <f>IFERROR(AVERAGEIF('Trade Journal'!O5:O54,"Loss",'Trade Journal'!N5:N54),0)</f>
         <v/>
       </c>
       <c r="F11" s="8" t="inlineStr">
@@ -2477,7 +2878,7 @@
         </is>
       </c>
       <c r="B12" s="16">
-        <f>IFERROR(MAX('Trade Journal'!M5:M54),0)</f>
+        <f>IFERROR(MAX('Trade Journal'!N5:N54),0)</f>
         <v/>
       </c>
       <c r="F12" s="6" t="inlineStr">
@@ -2486,7 +2887,7 @@
         </is>
       </c>
       <c r="G12" s="17">
-        <f>SUMPRODUCT((MONTH('Trade Journal'!A5:A54)=1)*('Trade Journal'!M5:M54))</f>
+        <f>SUMPRODUCT((MONTH('Trade Journal'!A5:A54)=1)*('Trade Journal'!N5:N54))</f>
         <v/>
       </c>
     </row>
@@ -2497,7 +2898,7 @@
         </is>
       </c>
       <c r="B13" s="16">
-        <f>IFERROR(MIN('Trade Journal'!M5:M54),0)</f>
+        <f>IFERROR(MIN('Trade Journal'!N5:N54),0)</f>
         <v/>
       </c>
       <c r="F13" s="4" t="inlineStr">
@@ -2506,7 +2907,7 @@
         </is>
       </c>
       <c r="G13" s="18">
-        <f>SUMPRODUCT((MONTH('Trade Journal'!A5:A54)=2)*('Trade Journal'!M5:M54))</f>
+        <f>SUMPRODUCT((MONTH('Trade Journal'!A5:A54)=2)*('Trade Journal'!N5:N54))</f>
         <v/>
       </c>
     </row>
@@ -2517,7 +2918,7 @@
         </is>
       </c>
       <c r="G14" s="17">
-        <f>SUMPRODUCT((MONTH('Trade Journal'!A5:A54)=3)*('Trade Journal'!M5:M54))</f>
+        <f>SUMPRODUCT((MONTH('Trade Journal'!A5:A54)=3)*('Trade Journal'!N5:N54))</f>
         <v/>
       </c>
     </row>
@@ -2533,7 +2934,7 @@
         </is>
       </c>
       <c r="G15" s="18">
-        <f>SUMPRODUCT((MONTH('Trade Journal'!A5:A54)=4)*('Trade Journal'!M5:M54))</f>
+        <f>SUMPRODUCT((MONTH('Trade Journal'!A5:A54)=4)*('Trade Journal'!N5:N54))</f>
         <v/>
       </c>
     </row>
@@ -2544,7 +2945,7 @@
         </is>
       </c>
       <c r="B16" s="20">
-        <f>COUNTIF('Trade Journal'!P5:P54,"No EMA Confirm")</f>
+        <f>COUNTIF('Trade Journal'!Q5:Q54,"No EMA Confirm")</f>
         <v/>
       </c>
       <c r="C16" s="21" t="n"/>
@@ -2555,7 +2956,7 @@
         </is>
       </c>
       <c r="G16" s="17">
-        <f>SUMPRODUCT((MONTH('Trade Journal'!A5:A54)=5)*('Trade Journal'!M5:M54))</f>
+        <f>SUMPRODUCT((MONTH('Trade Journal'!A5:A54)=5)*('Trade Journal'!N5:N54))</f>
         <v/>
       </c>
     </row>
@@ -2566,7 +2967,7 @@
         </is>
       </c>
       <c r="B17" s="22">
-        <f>COUNTIF('Trade Journal'!P5:P54,"Entered at S&amp;R")</f>
+        <f>COUNTIF('Trade Journal'!Q5:Q54,"Entered at S&amp;R")</f>
         <v/>
       </c>
       <c r="C17" s="23" t="n"/>
@@ -2577,7 +2978,7 @@
         </is>
       </c>
       <c r="G17" s="18">
-        <f>SUMPRODUCT((MONTH('Trade Journal'!A5:A54)=6)*('Trade Journal'!M5:M54))</f>
+        <f>SUMPRODUCT((MONTH('Trade Journal'!A5:A54)=6)*('Trade Journal'!N5:N54))</f>
         <v/>
       </c>
     </row>
@@ -2588,7 +2989,7 @@
         </is>
       </c>
       <c r="B18" s="20">
-        <f>COUNTIF('Trade Journal'!P5:P54,"RSI Extreme")</f>
+        <f>COUNTIF('Trade Journal'!Q5:Q54,"RSI Extreme")</f>
         <v/>
       </c>
       <c r="C18" s="21" t="n"/>
@@ -2599,7 +3000,7 @@
         </is>
       </c>
       <c r="G18" s="17">
-        <f>SUMPRODUCT((MONTH('Trade Journal'!A5:A54)=7)*('Trade Journal'!M5:M54))</f>
+        <f>SUMPRODUCT((MONTH('Trade Journal'!A5:A54)=7)*('Trade Journal'!N5:N54))</f>
         <v/>
       </c>
     </row>
@@ -2610,7 +3011,7 @@
         </is>
       </c>
       <c r="B19" s="22">
-        <f>COUNTIF('Trade Journal'!P5:P54,"Ignored OI")</f>
+        <f>COUNTIF('Trade Journal'!Q5:Q54,"Ignored OI")</f>
         <v/>
       </c>
       <c r="C19" s="23" t="n"/>
@@ -2621,7 +3022,7 @@
         </is>
       </c>
       <c r="G19" s="18">
-        <f>SUMPRODUCT((MONTH('Trade Journal'!A5:A54)=8)*('Trade Journal'!M5:M54))</f>
+        <f>SUMPRODUCT((MONTH('Trade Journal'!A5:A54)=8)*('Trade Journal'!N5:N54))</f>
         <v/>
       </c>
     </row>
@@ -2632,7 +3033,7 @@
         </is>
       </c>
       <c r="G20" s="17">
-        <f>SUMPRODUCT((MONTH('Trade Journal'!A5:A54)=9)*('Trade Journal'!M5:M54))</f>
+        <f>SUMPRODUCT((MONTH('Trade Journal'!A5:A54)=9)*('Trade Journal'!N5:N54))</f>
         <v/>
       </c>
     </row>
@@ -2643,7 +3044,7 @@
         </is>
       </c>
       <c r="G21" s="18">
-        <f>SUMPRODUCT((MONTH('Trade Journal'!A5:A54)=10)*('Trade Journal'!M5:M54))</f>
+        <f>SUMPRODUCT((MONTH('Trade Journal'!A5:A54)=10)*('Trade Journal'!N5:N54))</f>
         <v/>
       </c>
     </row>
@@ -2654,7 +3055,7 @@
         </is>
       </c>
       <c r="G22" s="17">
-        <f>SUMPRODUCT((MONTH('Trade Journal'!A5:A54)=11)*('Trade Journal'!M5:M54))</f>
+        <f>SUMPRODUCT((MONTH('Trade Journal'!A5:A54)=11)*('Trade Journal'!N5:N54))</f>
         <v/>
       </c>
     </row>
@@ -2665,17 +3066,193 @@
         </is>
       </c>
       <c r="G23" s="18">
-        <f>SUMPRODUCT((MONTH('Trade Journal'!A5:A54)=12)*('Trade Journal'!M5:M54))</f>
-        <v/>
-      </c>
+        <f>SUMPRODUCT((MONTH('Trade Journal'!A5:A54)=12)*('Trade Journal'!N5:N54))</f>
+        <v/>
+      </c>
+    </row>
+    <row r="26" ht="22" customHeight="1">
+      <c r="A26" s="40" t="inlineStr">
+        <is>
+          <t>STRATEGY COMPARISON — Intraday vs Swing</t>
+        </is>
+      </c>
+      <c r="B26" s="41" t="n"/>
+      <c r="C26" s="41" t="n"/>
+      <c r="D26" s="41" t="n"/>
+      <c r="E26" s="41" t="n"/>
+      <c r="F26" s="41" t="n"/>
+      <c r="G26" s="41" t="n"/>
+      <c r="H26" s="41" t="n"/>
+      <c r="I26" s="41" t="n"/>
+      <c r="J26" s="42" t="n"/>
+    </row>
+    <row r="27" ht="30" customHeight="1">
+      <c r="A27" s="38" t="inlineStr">
+        <is>
+          <t>Strategy</t>
+        </is>
+      </c>
+      <c r="B27" s="38" t="inlineStr">
+        <is>
+          <t>Total
+Trades</t>
+        </is>
+      </c>
+      <c r="C27" s="38" t="inlineStr">
+        <is>
+          <t>Wins</t>
+        </is>
+      </c>
+      <c r="D27" s="38" t="inlineStr">
+        <is>
+          <t>Losses</t>
+        </is>
+      </c>
+      <c r="E27" s="38" t="inlineStr">
+        <is>
+          <t>Win %</t>
+        </is>
+      </c>
+      <c r="F27" s="38" t="inlineStr">
+        <is>
+          <t>Total P&amp;L ₹</t>
+        </is>
+      </c>
+      <c r="G27" s="38" t="inlineStr">
+        <is>
+          <t>Avg Win ₹</t>
+        </is>
+      </c>
+      <c r="H27" s="38" t="inlineStr">
+        <is>
+          <t>Avg Loss ₹</t>
+        </is>
+      </c>
+      <c r="I27" s="38" t="inlineStr">
+        <is>
+          <t>Best Trade ₹</t>
+        </is>
+      </c>
+      <c r="J27" s="38" t="inlineStr">
+        <is>
+          <t>Worst Trade ₹</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="43" t="inlineStr">
+        <is>
+          <t>📊 Intraday</t>
+        </is>
+      </c>
+      <c r="B28" s="44">
+        <f>COUNTIF('Trade Journal'!B5:B54,"Intraday")</f>
+        <v/>
+      </c>
+      <c r="C28" s="44">
+        <f>COUNTIFS('Trade Journal'!B5:B54,"Intraday",'Trade Journal'!O5:O54,"Profit")</f>
+        <v/>
+      </c>
+      <c r="D28" s="44">
+        <f>COUNTIFS('Trade Journal'!B5:B54,"Intraday",'Trade Journal'!O5:O54,"Loss")</f>
+        <v/>
+      </c>
+      <c r="E28" s="45">
+        <f>IFERROR(C28/B28,0)</f>
+        <v/>
+      </c>
+      <c r="F28" s="46">
+        <f>SUMIF('Trade Journal'!B5:B54,"Intraday",'Trade Journal'!N5:N54)</f>
+        <v/>
+      </c>
+      <c r="G28" s="46">
+        <f>IFERROR(AVERAGEIFS('Trade Journal'!N5:N54,'Trade Journal'!B5:B54,"Intraday",'Trade Journal'!O5:O54,"Profit"),0)</f>
+        <v/>
+      </c>
+      <c r="H28" s="46">
+        <f>IFERROR(AVERAGEIFS('Trade Journal'!N5:N54,'Trade Journal'!B5:B54,"Intraday",'Trade Journal'!O5:O54,"Loss"),0)</f>
+        <v/>
+      </c>
+      <c r="I28" s="46">
+        <f>IFERROR(MAXIFS('Trade Journal'!N5:N54,'Trade Journal'!B5:B54,"Intraday"),0)</f>
+        <v/>
+      </c>
+      <c r="J28" s="46">
+        <f>IFERROR(MINIFS('Trade Journal'!N5:N54,'Trade Journal'!B5:B54,"Intraday"),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="47" t="inlineStr">
+        <is>
+          <t>📈 Swing</t>
+        </is>
+      </c>
+      <c r="B29" s="48">
+        <f>COUNTIF('Trade Journal'!B5:B54,"Swing")</f>
+        <v/>
+      </c>
+      <c r="C29" s="48">
+        <f>COUNTIFS('Trade Journal'!B5:B54,"Swing",'Trade Journal'!O5:O54,"Profit")</f>
+        <v/>
+      </c>
+      <c r="D29" s="48">
+        <f>COUNTIFS('Trade Journal'!B5:B54,"Swing",'Trade Journal'!O5:O54,"Loss")</f>
+        <v/>
+      </c>
+      <c r="E29" s="49">
+        <f>IFERROR(C29/B29,0)</f>
+        <v/>
+      </c>
+      <c r="F29" s="50">
+        <f>SUMIF('Trade Journal'!B5:B54,"Swing",'Trade Journal'!N5:N54)</f>
+        <v/>
+      </c>
+      <c r="G29" s="50">
+        <f>IFERROR(AVERAGEIFS('Trade Journal'!N5:N54,'Trade Journal'!B5:B54,"Swing",'Trade Journal'!O5:O54,"Profit"),0)</f>
+        <v/>
+      </c>
+      <c r="H29" s="50">
+        <f>IFERROR(AVERAGEIFS('Trade Journal'!N5:N54,'Trade Journal'!B5:B54,"Swing",'Trade Journal'!O5:O54,"Loss"),0)</f>
+        <v/>
+      </c>
+      <c r="I29" s="50">
+        <f>IFERROR(MAXIFS('Trade Journal'!N5:N54,'Trade Journal'!B5:B54,"Swing"),0)</f>
+        <v/>
+      </c>
+      <c r="J29" s="50">
+        <f>IFERROR(MINIFS('Trade Journal'!N5:N54,'Trade Journal'!B5:B54,"Swing"),0)</f>
+        <v/>
+      </c>
+    </row>
+    <row r="31" ht="22" customHeight="1">
+      <c r="A31" s="51" t="inlineStr">
+        <is>
+          <t>🏆 Better Strategy</t>
+        </is>
+      </c>
+      <c r="B31" s="52">
+        <f>IF(B28=0,"No Intraday trades yet",IF(B29=0,"No Swing trades yet",IF(E28&gt;E29,"📊 Intraday leads — Win Rate: "&amp;TEXT(E28,"0%")&amp;" vs "&amp;TEXT(E29,"0%"),"📈 Swing leads — Win Rate: "&amp;TEXT(E29,"0%")&amp;" vs "&amp;TEXT(E28,"0%"))))</f>
+        <v/>
+      </c>
+      <c r="C31" s="41" t="n"/>
+      <c r="D31" s="41" t="n"/>
+      <c r="E31" s="41" t="n"/>
+      <c r="F31" s="41" t="n"/>
+      <c r="G31" s="41" t="n"/>
+      <c r="H31" s="41" t="n"/>
+      <c r="I31" s="41" t="n"/>
+      <c r="J31" s="42" t="n"/>
     </row>
   </sheetData>
-  <mergeCells count="6">
+  <mergeCells count="8">
     <mergeCell ref="A1:J1"/>
     <mergeCell ref="F3:J3"/>
     <mergeCell ref="F11:J11"/>
     <mergeCell ref="A3:D3"/>
+    <mergeCell ref="B31:J31"/>
     <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A26:J26"/>
     <mergeCell ref="F4:J4"/>
   </mergeCells>
   <conditionalFormatting sqref="B9">
@@ -2744,6 +3321,10 @@
           <t>Check 15min chart first — price clearly above or below 21 EMA</t>
         </is>
       </c>
+      <c r="C4" s="53" t="n"/>
+      <c r="D4" s="53" t="n"/>
+      <c r="E4" s="53" t="n"/>
+      <c r="F4" s="54" t="n"/>
     </row>
     <row r="5" ht="20" customHeight="1">
       <c r="A5" s="26" t="inlineStr">
@@ -2756,6 +3337,10 @@
           <t>Confirm same direction on 1H chart (must agree with 15min)</t>
         </is>
       </c>
+      <c r="C5" s="53" t="n"/>
+      <c r="D5" s="53" t="n"/>
+      <c r="E5" s="53" t="n"/>
+      <c r="F5" s="54" t="n"/>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="26" t="inlineStr">
@@ -2768,6 +3353,10 @@
           <t>Confirm same direction on Daily chart (all 3 must align)</t>
         </is>
       </c>
+      <c r="C6" s="53" t="n"/>
+      <c r="D6" s="53" t="n"/>
+      <c r="E6" s="53" t="n"/>
+      <c r="F6" s="54" t="n"/>
     </row>
     <row r="7" ht="20" customHeight="1">
       <c r="A7" s="26" t="inlineStr">
@@ -2780,6 +3369,10 @@
           <t>All 3 EMA aligned BEARISH = only PE Buy or Call Sell</t>
         </is>
       </c>
+      <c r="C7" s="53" t="n"/>
+      <c r="D7" s="53" t="n"/>
+      <c r="E7" s="53" t="n"/>
+      <c r="F7" s="54" t="n"/>
     </row>
     <row r="8" ht="20" customHeight="1">
       <c r="A8" s="26" t="inlineStr">
@@ -2792,6 +3385,10 @@
           <t>All 3 EMA aligned BULLISH = only CE Buy or Put Sell</t>
         </is>
       </c>
+      <c r="C8" s="53" t="n"/>
+      <c r="D8" s="53" t="n"/>
+      <c r="E8" s="53" t="n"/>
+      <c r="F8" s="54" t="n"/>
     </row>
     <row r="9" ht="20" customHeight="1">
       <c r="A9" s="29" t="inlineStr">
@@ -2804,6 +3401,10 @@
           <t>If 3 timeframes conflict = NO TRADE</t>
         </is>
       </c>
+      <c r="C9" s="53" t="n"/>
+      <c r="D9" s="53" t="n"/>
+      <c r="E9" s="53" t="n"/>
+      <c r="F9" s="54" t="n"/>
     </row>
     <row r="11" ht="24" customHeight="1">
       <c r="A11" s="25" t="inlineStr">
@@ -2823,6 +3424,10 @@
           <t>Check RSI on 5min and 15min before every entry</t>
         </is>
       </c>
+      <c r="C12" s="53" t="n"/>
+      <c r="D12" s="53" t="n"/>
+      <c r="E12" s="53" t="n"/>
+      <c r="F12" s="54" t="n"/>
     </row>
     <row r="13" ht="20" customHeight="1">
       <c r="A13" s="26" t="inlineStr">
@@ -2835,6 +3440,10 @@
           <t>RSI near or below 30 (oversold) = WAIT. Do not buy PE. Wait for RSI to recover above 35</t>
         </is>
       </c>
+      <c r="C13" s="53" t="n"/>
+      <c r="D13" s="53" t="n"/>
+      <c r="E13" s="53" t="n"/>
+      <c r="F13" s="54" t="n"/>
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="A14" s="26" t="inlineStr">
@@ -2847,6 +3456,10 @@
           <t>RSI near or above 70 (overbought) = WAIT. Do not buy CE. Wait for RSI to pull back below 65</t>
         </is>
       </c>
+      <c r="C14" s="53" t="n"/>
+      <c r="D14" s="53" t="n"/>
+      <c r="E14" s="53" t="n"/>
+      <c r="F14" s="54" t="n"/>
     </row>
     <row r="15" ht="20" customHeight="1">
       <c r="A15" s="26" t="inlineStr">
@@ -2859,6 +3472,10 @@
           <t>RSI between 40-60 = neutral zone — best entries happen when RSI is moving directionally</t>
         </is>
       </c>
+      <c r="C15" s="53" t="n"/>
+      <c r="D15" s="53" t="n"/>
+      <c r="E15" s="53" t="n"/>
+      <c r="F15" s="54" t="n"/>
     </row>
     <row r="16" ht="20" customHeight="1">
       <c r="A16" s="31" t="inlineStr">
@@ -2871,6 +3488,10 @@
           <t>Price making lower low + RSI making higher low at support = Put Sell entry signal</t>
         </is>
       </c>
+      <c r="C16" s="53" t="n"/>
+      <c r="D16" s="53" t="n"/>
+      <c r="E16" s="53" t="n"/>
+      <c r="F16" s="54" t="n"/>
     </row>
     <row r="18" ht="24" customHeight="1">
       <c r="A18" s="25" t="inlineStr">
@@ -2890,6 +3511,10 @@
           <t>Mark key S&amp;R levels before market open using OI data and previous session levels</t>
         </is>
       </c>
+      <c r="C19" s="53" t="n"/>
+      <c r="D19" s="53" t="n"/>
+      <c r="E19" s="53" t="n"/>
+      <c r="F19" s="54" t="n"/>
     </row>
     <row r="20" ht="20" customHeight="1">
       <c r="A20" s="26" t="inlineStr">
@@ -2902,6 +3527,10 @@
           <t>NEVER enter when price is sitting at S&amp;R — wait for breakout or rejection</t>
         </is>
       </c>
+      <c r="C20" s="53" t="n"/>
+      <c r="D20" s="53" t="n"/>
+      <c r="E20" s="53" t="n"/>
+      <c r="F20" s="54" t="n"/>
     </row>
     <row r="21" ht="20" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
@@ -2914,6 +3543,10 @@
           <t>Rejection candle at resistance + EMA bearish = PE Buy entry</t>
         </is>
       </c>
+      <c r="C21" s="53" t="n"/>
+      <c r="D21" s="53" t="n"/>
+      <c r="E21" s="53" t="n"/>
+      <c r="F21" s="54" t="n"/>
     </row>
     <row r="22" ht="20" customHeight="1">
       <c r="A22" s="26" t="inlineStr">
@@ -2926,6 +3559,10 @@
           <t>Bounce + RSI divergence at support = Put Sell entry</t>
         </is>
       </c>
+      <c r="C22" s="53" t="n"/>
+      <c r="D22" s="53" t="n"/>
+      <c r="E22" s="53" t="n"/>
+      <c r="F22" s="54" t="n"/>
     </row>
     <row r="23" ht="20" customHeight="1">
       <c r="A23" s="26" t="inlineStr">
@@ -2938,6 +3575,10 @@
           <t>If price tested support 2-3 times = stronger bounce signal</t>
         </is>
       </c>
+      <c r="C23" s="53" t="n"/>
+      <c r="D23" s="53" t="n"/>
+      <c r="E23" s="53" t="n"/>
+      <c r="F23" s="54" t="n"/>
     </row>
     <row r="24" ht="20" customHeight="1">
       <c r="A24" s="29" t="inlineStr">
@@ -2950,6 +3591,10 @@
           <t>Price mid-range between S&amp;R = NO TRADE ZONE</t>
         </is>
       </c>
+      <c r="C24" s="53" t="n"/>
+      <c r="D24" s="53" t="n"/>
+      <c r="E24" s="53" t="n"/>
+      <c r="F24" s="54" t="n"/>
     </row>
     <row r="26" ht="24" customHeight="1">
       <c r="A26" s="25" t="inlineStr">
@@ -2969,6 +3614,10 @@
           <t>Check Sensibull OI data. Max Call OI strike = ceiling resistance</t>
         </is>
       </c>
+      <c r="C27" s="53" t="n"/>
+      <c r="D27" s="53" t="n"/>
+      <c r="E27" s="53" t="n"/>
+      <c r="F27" s="54" t="n"/>
     </row>
     <row r="28" ht="20" customHeight="1">
       <c r="A28" s="26" t="inlineStr">
@@ -2981,6 +3630,10 @@
           <t>Max Put OI strike = floor support. Never hold options against these walls</t>
         </is>
       </c>
+      <c r="C28" s="53" t="n"/>
+      <c r="D28" s="53" t="n"/>
+      <c r="E28" s="53" t="n"/>
+      <c r="F28" s="54" t="n"/>
     </row>
     <row r="29" ht="20" customHeight="1">
       <c r="A29" s="26" t="inlineStr">
@@ -2993,6 +3646,10 @@
           <t>PCR below 0.8 = bearish bias. PCR above 1.2 = bullish bias</t>
         </is>
       </c>
+      <c r="C29" s="53" t="n"/>
+      <c r="D29" s="53" t="n"/>
+      <c r="E29" s="53" t="n"/>
+      <c r="F29" s="54" t="n"/>
     </row>
     <row r="30" ht="20" customHeight="1">
       <c r="A30" s="26" t="inlineStr">
@@ -3005,6 +3662,10 @@
           <t>VIX rising sharply above 20 = avoid selling premium. High risk of loss</t>
         </is>
       </c>
+      <c r="C30" s="53" t="n"/>
+      <c r="D30" s="53" t="n"/>
+      <c r="E30" s="53" t="n"/>
+      <c r="F30" s="54" t="n"/>
     </row>
     <row r="31" ht="20" customHeight="1">
       <c r="A31" s="26" t="inlineStr">
@@ -3017,6 +3678,10 @@
           <t>OI must confirm chart direction. If they conflict = skip trade</t>
         </is>
       </c>
+      <c r="C31" s="53" t="n"/>
+      <c r="D31" s="53" t="n"/>
+      <c r="E31" s="53" t="n"/>
+      <c r="F31" s="54" t="n"/>
     </row>
     <row r="33" ht="24" customHeight="1">
       <c r="A33" s="33" t="inlineStr">
@@ -3036,6 +3701,10 @@
           <t>Minimum 1:2 Risk:Reward on every single trade — no exceptions</t>
         </is>
       </c>
+      <c r="C34" s="53" t="n"/>
+      <c r="D34" s="53" t="n"/>
+      <c r="E34" s="53" t="n"/>
+      <c r="F34" s="54" t="n"/>
     </row>
     <row r="35" ht="20" customHeight="1">
       <c r="A35" s="26" t="inlineStr">
@@ -3048,6 +3717,10 @@
           <t>Book 60% of position at Target 1. Trail SL to entry for balance</t>
         </is>
       </c>
+      <c r="C35" s="53" t="n"/>
+      <c r="D35" s="53" t="n"/>
+      <c r="E35" s="53" t="n"/>
+      <c r="F35" s="54" t="n"/>
     </row>
     <row r="36" ht="20" customHeight="1">
       <c r="A36" s="26" t="inlineStr">
@@ -3060,6 +3733,10 @@
           <t>Max 2 losing trades per day. If hit, stop trading immediately</t>
         </is>
       </c>
+      <c r="C36" s="53" t="n"/>
+      <c r="D36" s="53" t="n"/>
+      <c r="E36" s="53" t="n"/>
+      <c r="F36" s="54" t="n"/>
     </row>
     <row r="37" ht="20" customHeight="1">
       <c r="A37" s="26" t="inlineStr">
@@ -3072,6 +3749,10 @@
           <t>Never average a losing options position — exit at SL, reassess fresh</t>
         </is>
       </c>
+      <c r="C37" s="53" t="n"/>
+      <c r="D37" s="53" t="n"/>
+      <c r="E37" s="53" t="n"/>
+      <c r="F37" s="54" t="n"/>
     </row>
     <row r="38" ht="20" customHeight="1">
       <c r="A38" s="26" t="inlineStr">
@@ -3084,6 +3765,10 @@
           <t>Book profits before major S&amp;R levels. Never hold hoping for more</t>
         </is>
       </c>
+      <c r="C38" s="53" t="n"/>
+      <c r="D38" s="53" t="n"/>
+      <c r="E38" s="53" t="n"/>
+      <c r="F38" s="54" t="n"/>
     </row>
     <row r="39" ht="20" customHeight="1">
       <c r="A39" s="26" t="inlineStr">
@@ -3096,6 +3781,10 @@
           <t>1 lot only unless confidence is very high and setup is perfect</t>
         </is>
       </c>
+      <c r="C39" s="53" t="n"/>
+      <c r="D39" s="53" t="n"/>
+      <c r="E39" s="53" t="n"/>
+      <c r="F39" s="54" t="n"/>
     </row>
     <row r="41" ht="24" customHeight="1">
       <c r="A41" s="34" t="inlineStr">
@@ -3115,6 +3804,10 @@
           <t>Price at 23,800 or 23,900 support. Tested 2+ times already</t>
         </is>
       </c>
+      <c r="C42" s="53" t="n"/>
+      <c r="D42" s="53" t="n"/>
+      <c r="E42" s="53" t="n"/>
+      <c r="F42" s="54" t="n"/>
     </row>
     <row r="43" ht="20" customHeight="1">
       <c r="A43" s="31" t="inlineStr">
@@ -3127,6 +3820,10 @@
           <t>Price going down slowly (not crash). 5min RSI starts turning UP while price still flat/down</t>
         </is>
       </c>
+      <c r="C43" s="53" t="n"/>
+      <c r="D43" s="53" t="n"/>
+      <c r="E43" s="53" t="n"/>
+      <c r="F43" s="54" t="n"/>
     </row>
     <row r="44" ht="20" customHeight="1">
       <c r="A44" s="31" t="inlineStr">
@@ -3139,6 +3836,10 @@
           <t>Sell 23,850 PE or 23,750 PE after RSI curl confirmed on 5min</t>
         </is>
       </c>
+      <c r="C44" s="53" t="n"/>
+      <c r="D44" s="53" t="n"/>
+      <c r="E44" s="53" t="n"/>
+      <c r="F44" s="54" t="n"/>
     </row>
     <row r="45" ht="20" customHeight="1">
       <c r="A45" s="31" t="inlineStr">
@@ -3151,6 +3852,10 @@
           <t>Nifty spot breaks support level on closing basis (15min candle close)</t>
         </is>
       </c>
+      <c r="C45" s="53" t="n"/>
+      <c r="D45" s="53" t="n"/>
+      <c r="E45" s="53" t="n"/>
+      <c r="F45" s="54" t="n"/>
     </row>
     <row r="46" ht="20" customHeight="1">
       <c r="A46" s="31" t="inlineStr">
@@ -3163,6 +3868,10 @@
           <t>40-50% premium decay. Exit before VIX spikes or next session</t>
         </is>
       </c>
+      <c r="C46" s="53" t="n"/>
+      <c r="D46" s="53" t="n"/>
+      <c r="E46" s="53" t="n"/>
+      <c r="F46" s="54" t="n"/>
     </row>
     <row r="47" ht="20" customHeight="1">
       <c r="A47" s="31" t="inlineStr">
@@ -3175,6 +3884,10 @@
           <t>Do NOT Put Sell if: VIX &gt; 20, price crashing with big red candle, RSI still falling</t>
         </is>
       </c>
+      <c r="C47" s="53" t="n"/>
+      <c r="D47" s="53" t="n"/>
+      <c r="E47" s="53" t="n"/>
+      <c r="F47" s="54" t="n"/>
     </row>
     <row r="49" ht="24" customHeight="1">
       <c r="A49" s="35" t="inlineStr">
@@ -3194,6 +3907,10 @@
           <t>All 3 EMA timeframes confirmed in same direction?</t>
         </is>
       </c>
+      <c r="C50" s="53" t="n"/>
+      <c r="D50" s="53" t="n"/>
+      <c r="E50" s="53" t="n"/>
+      <c r="F50" s="54" t="n"/>
     </row>
     <row r="51" ht="20" customHeight="1">
       <c r="A51" s="26" t="inlineStr">
@@ -3206,6 +3923,10 @@
           <t>5min RSI not at extreme (below 30 or above 70)?</t>
         </is>
       </c>
+      <c r="C51" s="53" t="n"/>
+      <c r="D51" s="53" t="n"/>
+      <c r="E51" s="53" t="n"/>
+      <c r="F51" s="54" t="n"/>
     </row>
     <row r="52" ht="20" customHeight="1">
       <c r="A52" s="26" t="inlineStr">
@@ -3218,6 +3939,10 @@
           <t>15min RSI confirming direction (above/below 50)?</t>
         </is>
       </c>
+      <c r="C52" s="53" t="n"/>
+      <c r="D52" s="53" t="n"/>
+      <c r="E52" s="53" t="n"/>
+      <c r="F52" s="54" t="n"/>
     </row>
     <row r="53" ht="20" customHeight="1">
       <c r="A53" s="26" t="inlineStr">
@@ -3230,6 +3955,10 @@
           <t>Price NOT sitting at S&amp;R level?</t>
         </is>
       </c>
+      <c r="C53" s="53" t="n"/>
+      <c r="D53" s="53" t="n"/>
+      <c r="E53" s="53" t="n"/>
+      <c r="F53" s="54" t="n"/>
     </row>
     <row r="54" ht="20" customHeight="1">
       <c r="A54" s="26" t="inlineStr">
@@ -3242,6 +3971,10 @@
           <t>Entry is on rejection or confirmed breakout — not mid-zone?</t>
         </is>
       </c>
+      <c r="C54" s="53" t="n"/>
+      <c r="D54" s="53" t="n"/>
+      <c r="E54" s="53" t="n"/>
+      <c r="F54" s="54" t="n"/>
     </row>
     <row r="55" ht="20" customHeight="1">
       <c r="A55" s="26" t="inlineStr">
@@ -3254,6 +3987,10 @@
           <t>PCR and OI confirms chart direction?</t>
         </is>
       </c>
+      <c r="C55" s="53" t="n"/>
+      <c r="D55" s="53" t="n"/>
+      <c r="E55" s="53" t="n"/>
+      <c r="F55" s="54" t="n"/>
     </row>
     <row r="56" ht="20" customHeight="1">
       <c r="A56" s="26" t="inlineStr">
@@ -3266,6 +4003,10 @@
           <t>VIX not spiking above 20 (if selling)?</t>
         </is>
       </c>
+      <c r="C56" s="53" t="n"/>
+      <c r="D56" s="53" t="n"/>
+      <c r="E56" s="53" t="n"/>
+      <c r="F56" s="54" t="n"/>
     </row>
     <row r="57" ht="20" customHeight="1">
       <c r="A57" s="26" t="inlineStr">
@@ -3278,6 +4019,10 @@
           <t>Risk:Reward is at least 1:2?</t>
         </is>
       </c>
+      <c r="C57" s="53" t="n"/>
+      <c r="D57" s="53" t="n"/>
+      <c r="E57" s="53" t="n"/>
+      <c r="F57" s="54" t="n"/>
     </row>
     <row r="58" ht="20" customHeight="1">
       <c r="A58" s="31" t="inlineStr">
@@ -3290,6 +4035,10 @@
           <t>If all 8 = YES → Take trade. Any NO → Wait or skip</t>
         </is>
       </c>
+      <c r="C58" s="53" t="n"/>
+      <c r="D58" s="53" t="n"/>
+      <c r="E58" s="53" t="n"/>
+      <c r="F58" s="54" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="51">
@@ -3305,9 +4054,9 @@
     <mergeCell ref="B22:F22"/>
     <mergeCell ref="A3:F3"/>
     <mergeCell ref="A26:F26"/>
+    <mergeCell ref="B58:F58"/>
+    <mergeCell ref="B56:F56"/>
     <mergeCell ref="B27:F27"/>
-    <mergeCell ref="B56:F56"/>
-    <mergeCell ref="B58:F58"/>
     <mergeCell ref="B52:F52"/>
     <mergeCell ref="B21:F21"/>
     <mergeCell ref="A33:F33"/>
@@ -3388,6 +4137,11 @@
         </is>
       </c>
       <c r="B4" s="28" t="inlineStr"/>
+      <c r="C4" s="53" t="n"/>
+      <c r="D4" s="53" t="n"/>
+      <c r="E4" s="53" t="n"/>
+      <c r="F4" s="53" t="n"/>
+      <c r="G4" s="54" t="n"/>
     </row>
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="36" t="inlineStr">
@@ -3396,6 +4150,11 @@
         </is>
       </c>
       <c r="B5" s="28" t="inlineStr"/>
+      <c r="C5" s="53" t="n"/>
+      <c r="D5" s="53" t="n"/>
+      <c r="E5" s="53" t="n"/>
+      <c r="F5" s="53" t="n"/>
+      <c r="G5" s="54" t="n"/>
     </row>
     <row r="6" ht="22" customHeight="1">
       <c r="A6" s="36" t="inlineStr">
@@ -3408,6 +4167,11 @@
           <t>Positive / Negative / Neutral</t>
         </is>
       </c>
+      <c r="C6" s="53" t="n"/>
+      <c r="D6" s="53" t="n"/>
+      <c r="E6" s="53" t="n"/>
+      <c r="F6" s="53" t="n"/>
+      <c r="G6" s="54" t="n"/>
     </row>
     <row r="7" ht="22" customHeight="1">
       <c r="A7" s="36" t="inlineStr">
@@ -3416,6 +4180,11 @@
         </is>
       </c>
       <c r="B7" s="28" t="inlineStr"/>
+      <c r="C7" s="53" t="n"/>
+      <c r="D7" s="53" t="n"/>
+      <c r="E7" s="53" t="n"/>
+      <c r="F7" s="53" t="n"/>
+      <c r="G7" s="54" t="n"/>
     </row>
     <row r="8" ht="22" customHeight="1">
       <c r="A8" s="36" t="inlineStr">
@@ -3424,6 +4193,11 @@
         </is>
       </c>
       <c r="B8" s="28" t="inlineStr"/>
+      <c r="C8" s="53" t="n"/>
+      <c r="D8" s="53" t="n"/>
+      <c r="E8" s="53" t="n"/>
+      <c r="F8" s="53" t="n"/>
+      <c r="G8" s="54" t="n"/>
     </row>
     <row r="9" ht="22" customHeight="1">
       <c r="A9" s="36" t="inlineStr">
@@ -3432,6 +4206,11 @@
         </is>
       </c>
       <c r="B9" s="28" t="inlineStr"/>
+      <c r="C9" s="53" t="n"/>
+      <c r="D9" s="53" t="n"/>
+      <c r="E9" s="53" t="n"/>
+      <c r="F9" s="53" t="n"/>
+      <c r="G9" s="54" t="n"/>
     </row>
     <row r="10" ht="22" customHeight="1">
       <c r="A10" s="36" t="inlineStr">
@@ -3440,6 +4219,11 @@
         </is>
       </c>
       <c r="B10" s="28" t="inlineStr"/>
+      <c r="C10" s="53" t="n"/>
+      <c r="D10" s="53" t="n"/>
+      <c r="E10" s="53" t="n"/>
+      <c r="F10" s="53" t="n"/>
+      <c r="G10" s="54" t="n"/>
     </row>
     <row r="11" ht="22" customHeight="1">
       <c r="A11" s="36" t="inlineStr">
@@ -3448,6 +4232,11 @@
         </is>
       </c>
       <c r="B11" s="28" t="inlineStr"/>
+      <c r="C11" s="53" t="n"/>
+      <c r="D11" s="53" t="n"/>
+      <c r="E11" s="53" t="n"/>
+      <c r="F11" s="53" t="n"/>
+      <c r="G11" s="54" t="n"/>
     </row>
     <row r="12" ht="22" customHeight="1">
       <c r="A12" s="36" t="inlineStr">
@@ -3456,6 +4245,11 @@
         </is>
       </c>
       <c r="B12" s="28" t="inlineStr"/>
+      <c r="C12" s="53" t="n"/>
+      <c r="D12" s="53" t="n"/>
+      <c r="E12" s="53" t="n"/>
+      <c r="F12" s="53" t="n"/>
+      <c r="G12" s="54" t="n"/>
     </row>
     <row r="13" ht="22" customHeight="1">
       <c r="A13" s="36" t="inlineStr">
@@ -3468,6 +4262,11 @@
           <t>Bullish / Bearish / Sideways</t>
         </is>
       </c>
+      <c r="C13" s="53" t="n"/>
+      <c r="D13" s="53" t="n"/>
+      <c r="E13" s="53" t="n"/>
+      <c r="F13" s="53" t="n"/>
+      <c r="G13" s="54" t="n"/>
     </row>
     <row r="15" ht="24" customHeight="1">
       <c r="A15" s="25" t="inlineStr">
@@ -3483,6 +4282,11 @@
         </is>
       </c>
       <c r="B16" s="28" t="inlineStr"/>
+      <c r="C16" s="53" t="n"/>
+      <c r="D16" s="53" t="n"/>
+      <c r="E16" s="53" t="n"/>
+      <c r="F16" s="53" t="n"/>
+      <c r="G16" s="54" t="n"/>
     </row>
     <row r="17" ht="22" customHeight="1">
       <c r="A17" s="36" t="inlineStr">
@@ -3491,6 +4295,11 @@
         </is>
       </c>
       <c r="B17" s="28" t="inlineStr"/>
+      <c r="C17" s="53" t="n"/>
+      <c r="D17" s="53" t="n"/>
+      <c r="E17" s="53" t="n"/>
+      <c r="F17" s="53" t="n"/>
+      <c r="G17" s="54" t="n"/>
     </row>
     <row r="18" ht="22" customHeight="1">
       <c r="A18" s="36" t="inlineStr">
@@ -3499,6 +4308,11 @@
         </is>
       </c>
       <c r="B18" s="28" t="inlineStr"/>
+      <c r="C18" s="53" t="n"/>
+      <c r="D18" s="53" t="n"/>
+      <c r="E18" s="53" t="n"/>
+      <c r="F18" s="53" t="n"/>
+      <c r="G18" s="54" t="n"/>
     </row>
     <row r="19" ht="22" customHeight="1">
       <c r="A19" s="36" t="inlineStr">
@@ -3507,6 +4321,11 @@
         </is>
       </c>
       <c r="B19" s="28" t="inlineStr"/>
+      <c r="C19" s="53" t="n"/>
+      <c r="D19" s="53" t="n"/>
+      <c r="E19" s="53" t="n"/>
+      <c r="F19" s="53" t="n"/>
+      <c r="G19" s="54" t="n"/>
     </row>
     <row r="20" ht="22" customHeight="1">
       <c r="A20" s="36" t="inlineStr">
@@ -3515,6 +4334,11 @@
         </is>
       </c>
       <c r="B20" s="28" t="inlineStr"/>
+      <c r="C20" s="53" t="n"/>
+      <c r="D20" s="53" t="n"/>
+      <c r="E20" s="53" t="n"/>
+      <c r="F20" s="53" t="n"/>
+      <c r="G20" s="54" t="n"/>
     </row>
     <row r="21" ht="22" customHeight="1">
       <c r="A21" s="36" t="inlineStr">
@@ -3523,6 +4347,11 @@
         </is>
       </c>
       <c r="B21" s="28" t="inlineStr"/>
+      <c r="C21" s="53" t="n"/>
+      <c r="D21" s="53" t="n"/>
+      <c r="E21" s="53" t="n"/>
+      <c r="F21" s="53" t="n"/>
+      <c r="G21" s="54" t="n"/>
     </row>
     <row r="23" ht="24" customHeight="1">
       <c r="A23" s="25" t="inlineStr">
@@ -3538,6 +4367,11 @@
         </is>
       </c>
       <c r="B24" s="28" t="inlineStr"/>
+      <c r="C24" s="53" t="n"/>
+      <c r="D24" s="53" t="n"/>
+      <c r="E24" s="53" t="n"/>
+      <c r="F24" s="53" t="n"/>
+      <c r="G24" s="54" t="n"/>
     </row>
     <row r="25" ht="22" customHeight="1">
       <c r="A25" s="36" t="inlineStr">
@@ -3550,6 +4384,11 @@
           <t>PE Buy / CE Buy / Put Sell / Call Sell</t>
         </is>
       </c>
+      <c r="C25" s="53" t="n"/>
+      <c r="D25" s="53" t="n"/>
+      <c r="E25" s="53" t="n"/>
+      <c r="F25" s="53" t="n"/>
+      <c r="G25" s="54" t="n"/>
     </row>
     <row r="26" ht="22" customHeight="1">
       <c r="A26" s="36" t="inlineStr">
@@ -3558,6 +4397,11 @@
         </is>
       </c>
       <c r="B26" s="28" t="inlineStr"/>
+      <c r="C26" s="53" t="n"/>
+      <c r="D26" s="53" t="n"/>
+      <c r="E26" s="53" t="n"/>
+      <c r="F26" s="53" t="n"/>
+      <c r="G26" s="54" t="n"/>
     </row>
     <row r="27" ht="22" customHeight="1">
       <c r="A27" s="36" t="inlineStr">
@@ -3566,6 +4410,11 @@
         </is>
       </c>
       <c r="B27" s="28" t="inlineStr"/>
+      <c r="C27" s="53" t="n"/>
+      <c r="D27" s="53" t="n"/>
+      <c r="E27" s="53" t="n"/>
+      <c r="F27" s="53" t="n"/>
+      <c r="G27" s="54" t="n"/>
     </row>
     <row r="28" ht="22" customHeight="1">
       <c r="A28" s="36" t="inlineStr">
@@ -3574,6 +4423,11 @@
         </is>
       </c>
       <c r="B28" s="28" t="inlineStr"/>
+      <c r="C28" s="53" t="n"/>
+      <c r="D28" s="53" t="n"/>
+      <c r="E28" s="53" t="n"/>
+      <c r="F28" s="53" t="n"/>
+      <c r="G28" s="54" t="n"/>
     </row>
     <row r="29" ht="22" customHeight="1">
       <c r="A29" s="36" t="inlineStr">
@@ -3582,6 +4436,11 @@
         </is>
       </c>
       <c r="B29" s="28" t="inlineStr"/>
+      <c r="C29" s="53" t="n"/>
+      <c r="D29" s="53" t="n"/>
+      <c r="E29" s="53" t="n"/>
+      <c r="F29" s="53" t="n"/>
+      <c r="G29" s="54" t="n"/>
     </row>
     <row r="30" ht="22" customHeight="1">
       <c r="A30" s="36" t="inlineStr">
@@ -3590,6 +4449,11 @@
         </is>
       </c>
       <c r="B30" s="28" t="inlineStr"/>
+      <c r="C30" s="53" t="n"/>
+      <c r="D30" s="53" t="n"/>
+      <c r="E30" s="53" t="n"/>
+      <c r="F30" s="53" t="n"/>
+      <c r="G30" s="54" t="n"/>
     </row>
     <row r="31" ht="22" customHeight="1">
       <c r="A31" s="36" t="inlineStr">
@@ -3598,6 +4462,11 @@
         </is>
       </c>
       <c r="B31" s="28" t="inlineStr"/>
+      <c r="C31" s="53" t="n"/>
+      <c r="D31" s="53" t="n"/>
+      <c r="E31" s="53" t="n"/>
+      <c r="F31" s="53" t="n"/>
+      <c r="G31" s="54" t="n"/>
     </row>
     <row r="32" ht="22" customHeight="1">
       <c r="A32" s="36" t="inlineStr">
@@ -3606,6 +4475,11 @@
         </is>
       </c>
       <c r="B32" s="28" t="inlineStr"/>
+      <c r="C32" s="53" t="n"/>
+      <c r="D32" s="53" t="n"/>
+      <c r="E32" s="53" t="n"/>
+      <c r="F32" s="53" t="n"/>
+      <c r="G32" s="54" t="n"/>
     </row>
     <row r="34" ht="24" customHeight="1">
       <c r="A34" s="25" t="inlineStr">
@@ -3621,6 +4495,11 @@
         </is>
       </c>
       <c r="B35" s="28" t="inlineStr"/>
+      <c r="C35" s="53" t="n"/>
+      <c r="D35" s="53" t="n"/>
+      <c r="E35" s="53" t="n"/>
+      <c r="F35" s="53" t="n"/>
+      <c r="G35" s="54" t="n"/>
     </row>
     <row r="36" ht="22" customHeight="1">
       <c r="A36" s="36" t="inlineStr">
@@ -3629,6 +4508,11 @@
         </is>
       </c>
       <c r="B36" s="28" t="inlineStr"/>
+      <c r="C36" s="53" t="n"/>
+      <c r="D36" s="53" t="n"/>
+      <c r="E36" s="53" t="n"/>
+      <c r="F36" s="53" t="n"/>
+      <c r="G36" s="54" t="n"/>
     </row>
     <row r="37" ht="22" customHeight="1">
       <c r="A37" s="36" t="inlineStr">
@@ -3637,6 +4521,11 @@
         </is>
       </c>
       <c r="B37" s="28" t="inlineStr"/>
+      <c r="C37" s="53" t="n"/>
+      <c r="D37" s="53" t="n"/>
+      <c r="E37" s="53" t="n"/>
+      <c r="F37" s="53" t="n"/>
+      <c r="G37" s="54" t="n"/>
     </row>
     <row r="38" ht="22" customHeight="1">
       <c r="A38" s="36" t="inlineStr">
@@ -3645,6 +4534,11 @@
         </is>
       </c>
       <c r="B38" s="28" t="inlineStr"/>
+      <c r="C38" s="53" t="n"/>
+      <c r="D38" s="53" t="n"/>
+      <c r="E38" s="53" t="n"/>
+      <c r="F38" s="53" t="n"/>
+      <c r="G38" s="54" t="n"/>
     </row>
     <row r="39" ht="22" customHeight="1">
       <c r="A39" s="36" t="inlineStr">
@@ -3657,6 +4551,11 @@
           <t>Yes / No</t>
         </is>
       </c>
+      <c r="C39" s="53" t="n"/>
+      <c r="D39" s="53" t="n"/>
+      <c r="E39" s="53" t="n"/>
+      <c r="F39" s="53" t="n"/>
+      <c r="G39" s="54" t="n"/>
     </row>
     <row r="40" ht="22" customHeight="1">
       <c r="A40" s="36" t="inlineStr">
@@ -3665,6 +4564,11 @@
         </is>
       </c>
       <c r="B40" s="28" t="inlineStr"/>
+      <c r="C40" s="53" t="n"/>
+      <c r="D40" s="53" t="n"/>
+      <c r="E40" s="53" t="n"/>
+      <c r="F40" s="53" t="n"/>
+      <c r="G40" s="54" t="n"/>
     </row>
     <row r="41" ht="22" customHeight="1">
       <c r="A41" s="36" t="inlineStr">
@@ -3673,6 +4577,11 @@
         </is>
       </c>
       <c r="B41" s="28" t="inlineStr"/>
+      <c r="C41" s="53" t="n"/>
+      <c r="D41" s="53" t="n"/>
+      <c r="E41" s="53" t="n"/>
+      <c r="F41" s="53" t="n"/>
+      <c r="G41" s="54" t="n"/>
     </row>
     <row r="42" ht="22" customHeight="1">
       <c r="A42" s="36" t="inlineStr">
@@ -3681,6 +4590,11 @@
         </is>
       </c>
       <c r="B42" s="28" t="inlineStr"/>
+      <c r="C42" s="53" t="n"/>
+      <c r="D42" s="53" t="n"/>
+      <c r="E42" s="53" t="n"/>
+      <c r="F42" s="53" t="n"/>
+      <c r="G42" s="54" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="38">

</xml_diff>